<commit_message>
chore: update land law evaluation datasets and remove redundant question file
</commit_message>
<xml_diff>
--- a/emlaw_crawler/answer_dat_dai.xlsx
+++ b/emlaw_crawler/answer_dat_dai.xlsx
@@ -697,30 +697,48 @@
 Em có thửa đất được ba mẹ tặng cho năm 2010, có diện tích 200m2; kích thước ghi trong GCN là dài 33,33 và rộng 6m, chưa có tọa độ. Do không để ý nên giờ đo đạc thực tế thì còn dài dài 30m, rộng 6,2m diện tích 186m2. Em không có tranh chấp , đang là sổ hồng. Nhưng lên đính chính địa chính phường bảo là đã có sổ hồng thì không thể đính chính chiều ngang được, chỉ đính chính chiều dài giảm cho thực tế, chiều ngang vẫn 6m ghi trong GCN . Vậy cho em hỏi địa chính phường nói như vậy có đúng với luật đất đai không ? Cần làm gì để đính chính đúng với thực tế ?</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n"/>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Địa chính phường không thể kết luận chung rằng “đã có sổ hồng thì không được đính chính chiều ngang”. Nếu số đo ngang 6,2 m là ranh giới thực tế ổn định, không tranh chấp và phù hợp hồ sơ/hiện trạng quản lý đất, bạn có quyền yêu cầu cơ quan đăng ký đất đai kiểm tra, đo đạc lại để chỉnh lý đúng cả kích thước lẫn diện tích. Tuy nhiên, diện tích được công nhận còn phụ thuộc việc phần chênh lệch 14 m² có nằm trong ranh giới, nguồn gốc đất hợp pháp hay không.
+Việc đính chính được thực hiện khi Giấy chứng nhận có sai sót về thông tin thửa đất so với hồ sơ đăng ký đã được kiểm tra, xác nhận. Thông tin thửa đất bao gồm diện tích, ranh giới, kích thước; luật không có quy định chỉ được sửa chiều dài mà không được sửa chiều rộng. Điều 152 Luật Đất đai 2024
+Điểm cần phân biệt:
+Nếu thửa đất thực tế có ranh 6,2 m nhưng diện tích giảm xuống 186 m² vì chiều dài thực tế chỉ 30 m, cơ quan đo đạc cần xác định lại toàn bộ cạnh, mốc giới và diện tích thực. Sổ có thể được chỉnh lý theo kết quả đo đạc hợp pháp.
+Nếu 0,2 m chiều ngang là phần đất lấn sang thửa liền kề, đất công hoặc nằm ngoài ranh gốc, thì không được ghi nhận 6,2 m chỉ vì đang sử dụng thực tế.
+Nếu sổ năm 2010 ghi 200 m² nhưng đo đúng thực tế chỉ 186 m², không tranh chấp không đồng nghĩa đương nhiên được giữ nguyên 200 m². Cần đối chiếu hồ sơ tặng cho, hồ sơ cấp sổ, bản đồ/cắm mốc cũ và hiện trạng.
+Bạn nên làm như sau:
+Nộp đơn đề nghị đo đạc, xác định lại ranh giới, mốc giới thửa đất và đính chính Giấy chứng nhận tại Bộ phận một cửa cấp xã/phường hoặc Chi nhánh Văn phòng đăng ký đất đai nơi có đất. Yêu cầu trả lời bằng văn bản, không chỉ trả lời miệng.
+Kèm theo: bản gốc sổ hồng; CCCD; giấy tặng cho năm 2010 (nếu còn); trích đo hiện trạng hoặc biên bản đo đạc của đơn vị có chức năng (nếu đã có); ảnh mốc ranh; ý kiến/chữ ký xác nhận ranh giới của các chủ đất liền kề nếu có thể.
+Trong đơn, ghi rõ: đề nghị đo đạc chính quy; đối chiếu hồ sơ địa chính và hồ sơ cấp Giấy chứng nhận; xác định nguyên nhân chênh lệch; chỉnh lý đồng bộ “chiều dài, chiều rộng, diện tích và sơ đồ thửa đất” theo kết quả được cơ quan có thẩm quyền xác nhận.
+Nếu cơ quan tiếp nhận cho rằng không thể sửa ngang 6,2 m, yêu cầu họ nêu rõ căn cứ pháp luật, hồ sơ kỹ thuật hoặc ranh giới nào chứng minh 6,2 m không được công nhận. Nếu bị từ chối giải quyết, bạn có thể khiếu nại quyết định/hành vi hành chính đó.
+Bạn có thể dùng câu này trong đơn:
+“Kính đề nghị cơ quan có thẩm quyền tổ chức đo đạc địa chính, xác định ranh giới, mốc giới thửa đất; đối chiếu với hồ sơ đăng ký, hồ sơ cấp Giấy chứng nhận và thực tế sử dụng đất; thực hiện đính chính Giấy chứng nhận đối với toàn bộ thông tin kỹ thuật của thửa đất gồm kích thước các cạnh, diện tích và sơ đồ thửa đất, nếu xác định có sai sót theo quy định pháp luật.”
+Lưu ý: Đà Nẵng là địa phương có thủ tục tiếp nhận cụ thể, nhưng thẩm quyền quyết định kết quả đo đạc/đính chính thuộc cơ quan đăng ký đất đai có thẩm quyền, không phải cán bộ địa chính phường tự quyết định.
+[1]. Điều 152, Luật 31/2024/QH15</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Field answer rỗng (không có nội dung), không có gì để verify hay đánh giá.</t>
+          <t>Câu trả lời có trích dẫn Điều 152 của Luật Đất đai 2024 (Luật số 31/2024/QH15), tuy nhiên không có nội dung cụ thể của điều luật này được nêu ra trong câu trả lời. Điều này làm cho việc đánh giá tính đúng đắn và hiệu lực của điều luật trở nên khó khăn. Ngoài ra, câu trả lời không trích dẫn đầy đủ các quy định liên quan đến việc đính chính Giấy chứng nhận quyền sử dụng đất, chẳng hạn như các quy định về thủ tục và điều kiện đính chính. Do đó, tiêu chí trích dẫn điều luật được đánh giá là false.</t>
         </is>
       </c>
     </row>
@@ -786,30 +804,54 @@
 E có làm thủ tục cấp sổ lần đầu , tháng 1-7 e nộp tại uỷ ban và chuẩn bị đầy đủ giấy tờ theo cán bộ tiếp nhận hồ sơ yêu cầu . Đến 30-7 e nhận đc thông báo kết quả ( có văn bản trả lời ) là thiếu mất 3 hạng mục giấy tờ nữa . Lần tiếp theo là vào 5-12 e chuẩn bị đầy đủ các giấy tờ như trên văn bản yêu cầu , giấy hẹn trả kết quả là ngày 6-1 nhưng hiện tại e vẫn chưa nhận được kết quả , cũng thông cảm rằng khối lượng công việc họ nhiều có thể chậm 10 20 ngày nhưng e ra uỷ ban chỉ nhận được câu trả lời rằng đợi có tin nhắn về điện thoại . Vậy giờ chậm đến vài tháng không có tin nhắn mình cũng phải chịu ạ , và khi có kết quả lại thiếu cái nọ cái kia thì biết đến bao giờ mình mới hoàn tất đc hồ sơ . Nếu trường hợp e đã chuẩn bị đầy đủ hồ sơ như văn bản họ yêu cầu mà vẫn bị trả lại hồ sơ vì những lý do không đáng thì có e thể khởi kiện được không ạ , và nộp đơn ở những cơ quan nào ạ ? Xin các bác tư vấn , chỉ dẫn giúp e . E cảm ơn ạ</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n"/>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Bạn không phải chờ vô thời hạn chỉ vì “chưa có tin nhắn”. Nếu hồ sơ nộp ngày 05/12 đã đầy đủ theo phiếu yêu cầu bổ sung mà quá ngày hẹn 06/01 vẫn không có kết quả hoặc văn bản gia hạn/trả lời, bạn nên yêu cầu cơ quan tiếp nhận trả lời bằng văn bản; sau đó có thể khiếu nại hành vi chậm giải quyết hoặc khởi kiện hành chính.
+Thời hạn thủ tục cấp sổ lần đầu được tính từ khi cơ quan nhận hồ sơ đầy đủ, hợp lệ. Quy định trước đây tại Điều 22 Nghị định 101/2024/NĐ-CP đã bị sửa đổi bởi Nghị định 151/2025/NĐ-CP; vì vậy, cần căn cứ quy định đang áp dụng và thời hạn ghi trên phiếu hẹn/thủ tục công bố tại địa phương. Dù vậy, cơ quan giải quyết không được để hồ sơ kéo dài nhiều tháng mà không có thông báo chính thức về lý do, yêu cầu bổ sung hoặc gia hạn. Nghị định 101/2024/NĐ-CP
+Bạn nên làm ngay 3 việc:
+Nộp “Đơn đề nghị thông báo tình trạng và giải quyết hồ sơ đúng hạn” tại Bộ phận Một cửa nơi đã nhận hồ sơ. Đề nghị họ trả lời bằng văn bản về:
+Hồ sơ đã đầy đủ, hợp lệ hay chưa;
+Hồ sơ đang ở cơ quan/bộ phận nào;
+Lý do quá hạn;
+Thời điểm trả kết quả cụ thể;
+Nếu thiếu giấy tờ, phải nêu rõ từng giấy tờ, căn cứ pháp luật và chỉ yêu cầu bổ sung một lần đối với cùng nội dung.
+Giữ chứng cứ: phiếu tiếp nhận ngày 05/12, giấy hẹn 06/01, văn bản yêu cầu bổ sung ngày 30/07, giấy tờ đã nộp bổ sung, biên lai, ảnh/chụp màn hình tin nhắn (nếu có). Khi nộp đơn, yêu cầu đóng dấu đến hoặc lấy phiếu tiếp nhận.
+Nếu sau thời hạn yêu cầu hợp lý mà vẫn không giải quyết hoặc tiếp tục trả hồ sơ thiếu căn cứ, bạn có thể chọn:
+Khiếu nại lần đầu đến người đứng đầu cơ quan đang có hành vi chậm giải quyết hoặc ban hành văn bản trả hồ sơ; hoặc
+Khởi kiện vụ án hành chính tại Tòa án nhân dân có thẩm quyền đối với hành vi hành chính “không giải quyết/chậm giải quyết thủ tục hành chính” hay văn bản từ chối giải quyết trái pháp luật.
+Bạn không bắt buộc phải khiếu nại rồi mới được khởi kiện, trừ trường hợp pháp luật chuyên ngành quy định phải khiếu nại trước. Thời hiệu khởi kiện thông thường đối với quyết định hành chính, hành vi hành chính là 01 năm kể từ ngày nhận được/biết được quyết định hoặc hành vi đó. Điều 116 Luật Tố tụng hành chính 2015
+Nếu cơ quan trả hồ sơ lần nữa với lý do “không đáng”, bạn cần yêu cầu họ ban hành văn bản từ chối hoặc văn bản yêu cầu bổ sung ghi rõ căn cứ. Không nên chỉ nhận trả lời miệng, vì sẽ rất khó chứng minh khi khiếu nại hoặc khởi kiện.
+Mẫu nội dung ngắn để nộp:
+Tôi đã nộp hồ sơ đăng ký đất đai, cấp Giấy chứng nhận lần đầu ngày 05/12, giấy hẹn trả kết quả ngày 06/01. Hồ sơ đã được bổ sung theo văn bản yêu cầu trước đó. Nay đã quá hạn nhưng tôi chưa nhận được kết quả, thông báo gia hạn hoặc yêu cầu bổ sung bằng văn bản. Kính đề nghị cơ quan kiểm tra, thông báo tình trạng hồ sơ, lý do quá hạn và giải quyết/trả lời bằng văn bản theo quy định.
+Lưu ý: Trước khi khởi kiện, thường nên thực hiện khiếu nại bằng văn bản trước vì nhanh hơn, ít tốn kém hơn và giúp xác định rõ cơ quan nào đang giữ, chậm xử lý hồ sơ. Điều 7 Luật Khiếu nại 2011
+[1]. Nghị định 101/2024/NĐ-CP
+[2]. Điều 116, Luật 93/2015/QH13
+[3]. Điều 7, Luật 02/2011/QH13</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Field answer rỗng (không có nội dung), không có gì để verify hay đánh giá.</t>
+          <t>Câu trả lời trích dẫn Nghị định 101/2024/NĐ-CP và Điều 116 Luật Tố tụng hành chính 2015, Điều 7 Luật Khiếu nại 2011. Tuy nhiên, không có thông tin cụ thể về nội dung các điều luật này trong câu trả lời. Nghị định 101/2024/NĐ-CP là văn bản mới, nhưng không có thông tin chi tiết về nội dung điều luật liên quan đến thời hạn giải quyết hồ sơ cấp sổ lần đầu. Điều 116 Luật Tố tụng hành chính 2015 và Điều 7 Luật Khiếu nại 2011 là các điều luật còn hiệu lực và liên quan đến quyền khiếu nại và khởi kiện hành chính. Tuy nhiên, câu trả lời thiếu thông tin cụ thể về nội dung của các điều luật này và không trích dẫn điều luật cụ thể về thời hạn giải quyết hồ sơ cấp sổ lần đầu.</t>
         </is>
       </c>
     </row>
@@ -970,7 +1012,54 @@
 Thanks</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n"/>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Mẹ bạn chưa thể tự tách toàn bộ đất để chia cho 2 anh em nếu sổ đỏ là tài sản chung của bố mẹ hoặc đất đứng tên bố. Phần quyền sử dụng đất của bố phải được khai nhận/phân chia thừa kế trước; sau đó mẹ và những người thừa kế hợp pháp mới tặng cho hoặc phân chia để tách sổ cho hai bạn.
+Do bố mất đã 16 năm, nếu không có di chúc thì di sản của bố được chia theo pháp luật cho hàng thừa kế thứ nhất: mẹ bạn, các con của bố, và cha/mẹ của bố nếu họ còn sống tại thời điểm bố mất. Mỗi người cùng hàng hưởng phần bằng nhau. Thời hiệu yêu cầu chia di sản là bất động sản là 30 năm, nên hiện vẫn có thể làm thủ tục. Điều 651 Bộ luật Dân sự 2015 Điều 623 Bộ luật Dân sự 2015
+Ví dụ đất là tài sản chung vợ chồng: trước hết xác định mẹ có 1/2 thửa đất; 1/2 còn lại là di sản của bố và chia cho các đồng thừa kế nêu trên. Vì vậy, nếu chỉ có mẹ và 2 người con là người thừa kế thì mẹ thực tế có 2/3 thửa đất, mỗi người con có 1/6; không phải mẹ đương nhiên có toàn quyền chia cả thửa.
+Các bước thực hiện:
+Khai nhận hoặc thỏa thuận phân chia di sản thừa kế tại tổ chức công chứng. Tất cả người thừa kế của bố cần tham gia hoặc có văn bản từ chối nhận di sản/văn bản ủy quyền hợp lệ.
+Hồ sơ thường gồm: sổ đỏ; giấy chứng tử của bố; CCCD, giấy tờ cư trú; giấy khai sinh của các con; đăng ký kết hôn của bố mẹ; giấy tờ chứng minh cha mẹ của bố đã mất (nếu cần); giấy tờ về nguồn gốc đất.
+Tách thửa và đăng ký biến động/tặng cho. Sau khi xác định đủ người có quyền, các đồng thừa kế có thể lập văn bản thỏa thuận để đất được chia trực tiếp thành 2 phần cho hai người con, hoặc sang tên thừa kế trước rồi cùng lập hợp đồng tặng cho/phân chia. Tách thửa phải bảo đảm có sổ, không tranh chấp, còn thời hạn sử dụng, có lối đi phù hợp và đạt diện tích tối thiểu theo quy định của UBND tỉnh/thành nơi có đất. Điều 220 Luật Đất đai 2024
+Nộp hồ sơ tại Bộ phận Một cửa cấp xã hoặc Chi nhánh Văn phòng đăng ký đất đai nơi có đất để đo đạc/tách thửa, đăng ký biến động và cấp sổ mới.
+Nếu đất là tài sản riêng của mẹ (ví dụ mẹ được tặng cho riêng, thừa kế riêng; hoặc có căn cứ đất đã thuộc riêng mẹ), mẹ có thể trực tiếp làm thủ tục tách thửa rồi tặng cho 2 con mà không cần thủ tục thừa kế của bố. Ngược lại, nếu sổ chỉ đứng tên mẹ nhưng đất được tạo lập trong thời kỳ hôn nhân, vẫn cần kiểm tra nguồn gốc để tránh bỏ sót phần di sản của bố. Điều 33 Luật Hôn nhân và gia đình 2014
+Việc cha mẹ tặng cho quyền sử dụng đất cho con được miễn thuế thu nhập cá nhân và lệ phí trước bạ, nhưng vẫn có thể phát sinh phí công chứng, đo đạc, trích lục và phí cấp sổ. Điều 4 Luật Thuế thu nhập cá nhân 2007
+[1]. Điều 623, 651, Luật 91/2015/QH13
+[2]. Điều 220, Luật 31/2024/QH15
+[3]. Điều 33, Luật 52/2014/QH13
+[4]. Điều 4, Luật 04/2007/QH12</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Câu trả lời đã trích dẫn các điều luật sau:
+1. Điều 623, 651 Bộ luật Dân sự 2015: Các điều này liên quan đến thừa kế theo pháp luật và thời hiệu thừa kế. Các điều luật này còn hiệu lực và phù hợp với tình huống.
+2. Điều 220 Luật Đất đai 2024: Điều này liên quan đến việc tách thửa đất. Điều luật này còn hiệu lực và phù hợp với tình huống.
+3. Điều 33 Luật Hôn nhân và gia đình 2014: Điều này liên quan đến tài sản chung và riêng của vợ chồng. Điều luật này còn hiệu lực và phù hợp với tình huống.
+4. Điều 4 Luật Thuế thu nhập cá nhân 2007: Điều này liên quan đến miễn thuế thu nhập cá nhân khi tặng cho giữa cha mẹ và con cái. Điều luật này còn hiệu lực và phù hợp với tình huống.
+Tuy nhiên, câu trả lời đã sử dụng Luật Đất đai 2013 (Luật số 45/2013/QH13) và các nghị định cũ đã hết hiệu lực, điều này vi phạm tiêu chí về tính hiệu lực của điều luật.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="409.6" customHeight="1">
       <c r="A13" s="2" t="n">
@@ -1129,7 +1218,51 @@
 Giờ em kiện thì có đòi được không? Và kiện ai</t>
         </is>
       </c>
-      <c r="C19" s="2" t="n"/>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Bạn có cơ sở để yêu cầu hoàn lại tiền cọc nếu môi giới tự ký hợp đồng cọc nhân danh bạn mà không có quyền đại diện và bạn chưa công nhận giao dịch đó. Trước mắt, nên yêu cầu cả môi giới và chủ đất cung cấp hợp đồng cọc, chứng từ giao tiền; nếu không giải quyết, có thể khởi kiện dân sự, thường nên đưa cả hai vào vụ án để Tòa xác định đúng người phải hoàn tiền.
+Người không có quyền đại diện ký thay người khác thì giao dịch không làm phát sinh nghĩa vụ cho người bị đại diện, trừ khi người đó đã công nhận giao dịch, biết mà không phản đối trong thời gian hợp lý, hoặc có lỗi làm bên kia tin rằng người ký có quyền. Điều 142 Bộ luật Dân sự 2015
+Vì bạn là người trực tiếp chuyển tiền cho môi giới để “cọc hộ”, chủ đất có thể lập luận rằng bạn đã ủy quyền bằng hành vi. Do đó, việc không có giấy ủy quyền hoặc tin nhắn chưa chắc giúp bạn đòi lại được tiền. Tòa sẽ xem toàn bộ chứng cứ: nội dung chuyển khoản, tin nhắn/cuộc gọi, bạn có biết việc môi giới ký thay không, hợp đồng cọc ghi ai là bên đặt cọc, chủ đất có biết môi giới không có quyền hay không.
+Mâu thuẫn vợ chồng và không mua được nữa thường được xem là lý do từ phía bên mua. Nếu hợp đồng cọc hợp lệ và bạn được xác định là bên đặt cọc, chủ đất có quyền giữ cọc khi bạn từ chối mua, trừ khi hợp đồng có thỏa thuận khác. Điều 328 Bộ luật Dân sự 2015
+Bạn nên làm ngay:
+Yêu cầu môi giới gửi bản hợp đồng cọc có chữ ký; chứng từ đã chuyển tiền cọc cho chủ đất; tin nhắn/chứng cứ chủ đất chấp nhận việc môi giới đại diện bạn.
+Gửi văn bản hoặc tin nhắn có thể lưu chứng cứ cho cả môi giới và chủ đất: “Tôi không ủy quyền cho anh/chị ký hợp đồng đặt cọc nhân danh tôi; không công nhận hợp đồng này; đề nghị hoàn trả số tiền… trong … ngày.” Không ký thêm giấy xác nhận, biên bản thanh lý hay giấy chịu mất cọc nếu chưa xem kỹ.
+Lưu sao kê chuyển khoản, nội dung trao đổi, ghi âm hợp pháp các trao đổi mà bạn là người tham gia, quảng cáo môi giới, thông tin người làm chứng.
+Kiện ai?
+Bạn có thể khởi kiện:
+Môi giới, nếu họ tự ý ký, cam kết thay bạn hoặc giữ/nhận tiền của bạn không đúng thỏa thuận;
+Chủ đất, nếu họ đang giữ tiền cọc và biết hoặc phải biết môi giới không có quyền đại diện;
+Thực tế nên ghi cả môi giới và chủ đất là người có quyền lợi, nghĩa vụ liên quan hoặc đồng bị đơn tùy yêu cầu cụ thể, để Tòa làm rõ tiền đang ở đâu, hợp đồng có ràng buộc bạn không và ai phải trả.
+Đơn kiện nộp tại Tòa án nhân dân khu vực nơi bị đơn cư trú/làm việc; nếu yêu cầu chính gắn trực tiếp với tranh chấp hợp đồng về quyền sử dụng thửa đất cụ thể, có thể thuộc Tòa án nơi có đất. Bạn cần kèm hợp đồng cọc (nếu có), sao kê chuyển tiền, toàn bộ tin nhắn và văn bản yêu cầu hoàn tiền.
+Lưu ý quan trọng: nếu chứng cứ cho thấy bạn đã nhờ môi giới cọc hộ, biết họ ký thay và chỉ đổi ý sau đó, khả năng lấy lại cọc sẽ thấp. Ngược lại, nếu môi giới tự quyết việc ký cọc, tự cam kết điều khoản/phạt cọc vượt quá sự đồng ý của bạn, hoặc không chứng minh đã giao tiền cho chủ đất, bạn có cơ sở yêu cầu môi giới hoàn trả và bồi thường thiệt hại nếu có.
+[1]. Điều 142, 328, Luật 91/2015/QH13</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Điều 142 và 328 của Bộ luật Dân sự 2015 (Luật 91/2015/QH13). Tuy nhiên, các điều luật này vẫn còn hiệu lực và đúng với vấn đề pháp lý được hỏi. Tuy nhiên, câu trả lời không trích dẫn các điều luật mới nhất liên quan đến Luật Đất đai 2024 và các nghị định mới, do đó không đáp ứng đầy đủ yêu cầu về tính hiệu lực hiện hành của các văn bản pháp luật liên quan đến đất đai.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="224" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -1145,7 +1278,62 @@
 Em cảm ơn</t>
         </is>
       </c>
-      <c r="C20" s="2" t="n"/>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Gia đình bạn không nên ký biên bản có nội dung đồng ý cưỡng chế hoặc tự nguyện bàn giao đất khi chưa nhận được đầy đủ hồ sơ thu hồi đất và phương án bồi thường. Việc xã nói “sau 3 ngày sẽ cưỡng chế” chưa đủ căn cứ để cưỡng chế hợp pháp nếu chưa có quyết định thu hồi đất, quyết định cưỡng chế bằng văn bản và chưa bảo đảm điều kiện, trình tự luật định.
+Gia đình có thể được bồi thường về đất nếu chứng minh đất 30 m² đang sử dụng ổn định, không tranh chấp và đủ điều kiện được cấp Giấy chứng nhận theo pháp luật đất đai, dù hiện chưa có sổ và chưa đóng thuế. Nếu không đủ điều kiện bồi thường về đất, vẫn cần xem xét bồi thường cây trồng, chi phí đầu tư vào đất còn lại và các khoản hỗ trợ theo phương án được phê duyệt.
+1. Yêu cầu xã cung cấp các giấy tờ sau
+Bạn nên nộp đơn yêu cầu UBND xã/cơ quan thực hiện dự án cung cấp hoặc cho sao chụp:
+Thông báo thu hồi đất;
+Quyết định thu hồi đất đối với diện tích 30 m²;
+Bản đồ, trích đo xác định chính xác phần đất bị ảnh hưởng;
+Phương án bồi thường, hỗ trợ đã được niêm yết và phê duyệt;
+Biên bản kiểm đếm cây ăn quả, tài sản trên đất;
+Nếu có: quyết định cưỡng chế thu hồi đất.
+Không ký biên bản nếu nội dung ghi “tự nguyện hiến đất”, “đồng ý không nhận bồi thường”, “đồng ý bàn giao” hoặc xác nhận số liệu không đúng. Nếu cần ký để xác nhận đã nhận giấy tờ, ghi tay: “Chỉ xác nhận đã nhận/đã được thông báo; không đồng ý việc không bồi thường và bảo lưu quyền khiếu nại.”
+2. Cưỡng chế không thể chỉ dựa vào giấy triệu tập
+Cưỡng chế thu hồi đất chỉ được thực hiện khi có quyết định cưỡng chế của người có thẩm quyền, đã được giao hợp lệ; người bị thu hồi không chấp hành quyết định thu hồi đất sau khi được vận động, thuyết phục; và phải đáp ứng các điều kiện, trình tự cưỡng chế. Hành vi cưỡng chế không đúng điều kiện, nguyên tắc, thẩm quyền hoặc thủ tục là vi phạm pháp luật. Điều 109 Nghị định 102/2024/NĐ-CP
+Vì vậy, việc nói miệng rằng “03 ngày không dời cây thì sẽ cưỡng chế” không thay thế được quyết định cưỡng chế bằng văn bản. Bạn cần yêu cầu họ cho biết: ai ký quyết định, số quyết định, ngày ban hành, phạm vi cưỡng chế và thời điểm thực hiện.
+3. Về khả năng được bồi thường
+Không có giấy tờ, không đóng thuế không đồng nghĩa chắc chắn không được bồi thường. Cần xác minh nguồn gốc “các cụ để lại”, thời điểm gia đình bắt đầu sử dụng, việc sử dụng có liên tục/công khai hay không, có ai tranh chấp không và đất có thuộc quỹ đất công, đất công ích hoặc hành lang công trình hay không.
+Gia đình nên xin UBND xã xác nhận bằng văn bản về: thời điểm sử dụng đất; nguồn gốc do ông bà/cụ để lại; sử dụng ổn định; không tranh chấp; hiện trạng trồng cây ăn quả; có hay không việc đất thuộc quỹ đất công ích. Đây là chứng cứ quan trọng để cơ quan bồi thường xem xét điều kiện bồi thường về đất.
+Dù chưa được bồi thường về đất, cây ăn quả có trước thời điểm thông báo thu hồi đất phải được kiểm đếm và xử lý trong phương án bồi thường, hỗ trợ. Không tự chặt phá, di dời cây trước khi có biên bản kiểm đếm đầy đủ, trừ trường hợp cần thiết và đã lập chứng cứ về hiện trạng.
+4. Cách phản đối đúng thủ tục
+Trong thời gian sớm nhất, gửi “Đơn đề nghị xác định nguồn gốc đất, kiểm đếm tài sản và xem xét bồi thường, hỗ trợ khi thu hồi đất” đến UBND xã, cơ quan thực hiện bồi thường/giải phóng mặt bằng và UBND cấp có thẩm quyền thu hồi đất. Nộp tại bộ phận một cửa và giữ phiếu nhận đơn.
+Nếu đã có quyết định thu hồi đất hoặc phương án bồi thường nhưng bạn cho rằng sai, bạn có thể khiếu nại người đã ban hành quyết định. Người dân được lựa chọn khiếu nại hoặc khởi kiện vụ án hành chính; thời hiệu khởi kiện thông thường là 01 năm từ ngày nhận được hoặc biết được quyết định, hành vi hành chính. Điều 7 Luật Khiếu nại 2011 Điều 116 Luật Tố tụng hành chính 2015
+Bạn có thể ghi ngắn trong đơn:
+Gia đình tôi đang sử dụng ổn định diện tích khoảng 30 m² đất trồng cây ăn quả do tổ tiên để lại, không có tranh chấp. Đề nghị cơ quan có thẩm quyền xác minh nguồn gốc, thời điểm sử dụng đất; tổ chức đo đạc, kiểm đếm toàn bộ cây trồng/tài sản; cung cấp quyết định thu hồi đất, phương án bồi thường hỗ trợ và xem xét bồi thường theo quy định. Gia đình không đồng ý cưỡng chế khi chưa được cung cấp đầy đủ hồ sơ, chưa kiểm đếm và chưa giải quyết ý kiến về bồi thường.
+Do bạn chưa nêu tỉnh/thành phố nơi có đất, chưa thể xác định mức giá cây trồng, mức hỗ trợ và quy định bồi thường cụ thể của địa phương.
+[1]. Điều 109, Nghị định 102/2024/NĐ-CP
+[2]. Điều 7, Luật 02/2011/QH13
+[3]. Điều 116, Luật 93/2015/QH13</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Điều 109 Nghị định 102/2024/NĐ-CP về cưỡng chế thu hồi đất, Điều 7 Luật Khiếu nại 2011 và Điều 116 Luật Tố tụng hành chính 2015. Tuy nhiên, Nghị định 102/2024/NĐ-CP là văn bản mới và có thể chưa được phổ biến rộng rãi, cần kiểm tra lại tính chính xác của nội dung trích dẫn. Các điều luật khác được trích dẫn đúng và còn hiệu lực. Câu trả lời đã bao phủ phần lớn các khía cạnh pháp lý liên quan đến cưỡng chế và bồi thường đất, nhưng cần thêm thông tin cụ thể về điều kiện bồi thường theo Luật Đất đai 2024.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="409.6" customHeight="1">
       <c r="A21" s="2" t="n">
@@ -1328,7 +1516,52 @@
 mọi người có hướng nào giải quyết không ạ</t>
         </is>
       </c>
-      <c r="C28" s="2" t="n"/>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Hồ sơ đổi/cấp lại sổ đã kéo dài 7 tháng mà không có văn bản nêu rõ lý do là bất thường. Bạn nên yêu cầu cơ quan tiếp nhận trả lời bằng văn bản về tình trạng hồ sơ, lý do quá hạn và thời hạn xử lý; nếu tiếp tục chậm, thực hiện khiếu nại hoặc khởi kiện hành chính.
+Đầu tiên, xác định bạn đang làm thủ tục nào: cấp đổi Giấy chứng nhận (sổ cũ rách, sai thông tin, cần đổi mẫu), đính chính, hay cấp lại do mất. Mỗi thủ tục có thành phần và thời hạn khác nhau; cán bộ địa chính xã/phường chủ yếu xác minh hoặc chuyển hồ sơ, còn cơ quan đăng ký đất đai có trách nhiệm xử lý, trả kết quả. Việc “làm khó” bằng yêu cầu miệng không phải căn cứ hợp lệ.
+Bạn nên nộp một đơn ngắn tại Bộ phận Một cửa nơi đã nộp hồ sơ, yêu cầu:
+Cung cấp số hồ sơ, bộ phận/cơ quan đang thụ lý;
+Xác nhận hồ sơ đầy đủ hay thiếu giấy tờ nào;
+Nếu thiếu, phải yêu cầu bằng văn bản, ghi rõ căn cứ pháp luật;
+Nêu lý do quá hạn và ngày trả kết quả cụ thể.
+Kèm bản sao phiếu tiếp nhận, giấy hẹn, sổ cũ và toàn bộ chứng từ đã nộp. Khi nộp đơn, yêu cầu đóng dấu nhận hoặc cấp phiếu tiếp nhận. Thủ tục cấp đổi Giấy chứng nhận được thực hiện theo quy định về đăng ký đất đai, cấp Giấy chứng nhận; cơ quan tiếp nhận phải hướng dẫn hồ sơ đầy đủ, rõ ràng. Nghị định 101/2024/NĐ-CP
+Nếu có văn bản từ chối, yêu cầu bổ sung không có căn cứ, hoặc tiếp tục không giải quyết, bạn có thể:
+Khiếu nại lần đầu đến người đứng đầu cơ quan đang thụ lý/chậm giải quyết hồ sơ;
+Hoặc khởi kiện tại Tòa án nhân dân có thẩm quyền đối với hành vi hành chính chậm giải quyết. Người dân có quyền chọn khiếu nại hoặc khởi kiện; thời hiệu khởi kiện thông thường là 01 năm kể từ ngày biết hành vi hành chính. Điều 7 Luật Khiếu nại 2011 Điều 116 Luật Tố tụng hành chính 2015
+Bạn có thể ghi trong đơn:
+Tôi nộp hồ sơ … ngày …, số hồ sơ …, hẹn trả ngày … nhưng đến nay chưa nhận được kết quả hoặc thông báo bằng văn bản. Kính đề nghị cơ quan kiểm tra, thông báo tình trạng hồ sơ, lý do quá hạn và giải quyết/trả lời bằng văn bản theo quy định.
+Nếu bạn cho biết đất ở tỉnh/thành nào, đã nộp hồ sơ tại đâu và loại thủ tục ghi trên phiếu hẹn, tôi có thể chỉ đúng cơ quan nhận khiếu nại và hướng xử lý sát hồ sơ hơn.
+[1]. Nghị định 101/2024/NĐ-CP
+[2]. Điều 7, Luật 02/2011/QH13
+[3]. Điều 116, Luật 93/2015/QH13</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Câu trả lời có trích dẫn Nghị định 101/2024/NĐ-CP, Điều 7 Luật Khiếu nại 2011 và Điều 116 Luật Tố tụng hành chính 2015. Tuy nhiên, không có thông tin cụ thể về nội dung các điều luật này trong câu trả lời. Ngoài ra, Luật Khiếu nại 2011 và Luật Tố tụng hành chính 2015 vẫn còn hiệu lực, nhưng cần kiểm tra tính chính xác của các điều luật cụ thể được trích dẫn. Câu trả lời chưa trích dẫn điều luật cụ thể nào từ Luật Đất đai 2024 liên quan đến thủ tục cấp đổi Giấy chứng nhận, điều này làm giảm mức độ bao phủ của câu trả lời.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="409.6" customHeight="1">
       <c r="A29" s="2" t="n">
@@ -1397,7 +1630,54 @@
 Xin hỏi trong trường hợp đất khai hoang, sử dụng ổn định lâu dài như vậy thì gia đình tôi có hướng giải quyết pháp lý nào không? Cần làm những thủ tục gì để bảo vệ quyền lợi?</t>
         </is>
       </c>
-      <c r="C31" s="2" t="n"/>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Gia đình bạn vẫn có hướng bảo vệ quyền lợi, nhưng không thể chỉ nộp hồ sơ xin cấp sổ ngay vì phần đất đang có tranh chấp và hồ sơ địa chính đang ghi tên chú. Cần làm rõ bằng chứng cha mẹ là người khai hoang, quản lý, sử dụng thực tế; trước hết hòa giải tranh chấp tại UBND cấp xã, không thành thì khởi kiện tại Tòa án để yêu cầu xác định quyền sử dụng đất.
+Việc chú đứng tên trên hồ sơ địa chính không tự động chứng minh chú là người có quyền sử dụng đất hợp pháp; đó là một chứng cứ để xem xét cùng với nguồn gốc, quá trình quản lý, sử dụng đất và hồ sơ đăng ký ban đầu. Tuy nhiên, gia đình bạn phải chứng minh việc “nhờ đứng tên” là có thật, đồng thời chứng minh cha mẹ đã khai hoang, sử dụng đất công khai, liên tục, ổn định từ trước đến nay.
+Các chứng cứ nên thu thập gồm:
+Giấy tờ xin phép địa phương làm nhà, khai phá hoặc sử dụng đất trước đây;
+Biên lai thuế, nghĩa vụ tài chính, giấy đăng ký nhà/điện/nước, hồ sơ cư trú gắn với thửa đất;
+Ảnh cũ, giấy tờ xây dựng, cây trồng, công trình do gia đình tạo lập;
+Văn bản hoặc người làm chứng là hàng xóm, tổ trưởng/thôn, cán bộ cũ về việc cha mẹ khai hoang và sử dụng liên tục;
+Hồ sơ địa chính thể hiện thời điểm, căn cứ nào ghi chú là người sử dụng đất;
+Tin nhắn, ghi âm hợp pháp, giấy tờ thể hiện chú thừa nhận chỉ đứng tên giúp.
+Hướng xử lý theo trình tự
+Gửi đơn yêu cầu UBND cấp xã xác minh nguồn gốc, thời điểm sử dụng, hiện trạng và tổ chức hòa giải tranh chấp đất đai. Đơn cần đề nghị sao lục/xác nhận các tài liệu địa chính có tên chú: sổ mục kê, sổ địa chính, bản đồ, đơn đăng ký, biên bản xét duyệt, tài liệu kê khai của chú.
+Nếu hòa giải thành, lập văn bản hòa giải thành hoặc văn bản thỏa thuận xác định quyền sử dụng đất; sau đó thực hiện đăng ký biến động/cấp Giấy chứng nhận theo kết quả hòa giải và hồ sơ đất đai.
+Nếu hòa giải không thành, yêu cầu UBND xã lập biên bản hòa giải không thành. Đây là điều kiện bắt buộc trước khi khởi kiện tranh chấp về ai có quyền sử dụng đất tại Tòa án. Điều 235 Luật Đất đai 2024
+Khởi kiện tại Tòa án nhân dân có thẩm quyền nơi có đất, yêu cầu: xác định quyền sử dụng gần 1.000 m² đất thuộc cha mẹ/gia đình bạn; hủy hoặc điều chỉnh thông tin địa chính ghi tên chú nếu việc ghi nhận không đúng; buộc chú chấm dứt cản trở thủ tục đăng ký đất đai. Nếu cha hoặc mẹ đã mất, cần xác định những người thừa kế và đưa họ tham gia vụ án.
+Về khả năng được cấp sổ: người đang sử dụng đất không có giấy tờ có thể được xem xét cấp Giấy chứng nhận nếu đáp ứng điều kiện về sử dụng ổn định, không vi phạm pháp luật đất đai, không thuộc trường hợp giao đất trái thẩm quyền và phù hợp quy hoạch theo từng trường hợp. Nhưng do hiện có tranh chấp với chú, cơ quan đăng ký đất đai thường sẽ không cấp sổ cho đến khi tranh chấp được giải quyết xong. Điều 138 Luật Đất đai 2024
+Không nên lập giấy ủy quyền để chú “ủy quyền lại” cho gia đình làm sổ nếu chú không thừa nhận quyền của gia đình; giấy ủy quyền chỉ cho phép thực hiện công việc, không giải quyết dứt điểm việc ai là chủ sử dụng đất. Phương án tốt nhất là đề nghị chú ký văn bản xác nhận nguồn gốc và thỏa thuận chuyển giao/xác lập quyền sử dụng đất, có công chứng nếu đủ điều kiện; nếu chú không hợp tác thì đi theo con đường hòa giải và Tòa án.
+Trong đơn hòa giải, bạn có thể nêu ngắn:
+Cha mẹ tôi là người trực tiếp khai hoang, bao đất, xây nhà và sử dụng ổn định, công khai đối với diện tích khoảng … m² từ năm …; chú … chỉ đứng tên kê khai/hồ sơ địa chính theo sự nhờ vả, không trực tiếp quản lý sử dụng. Nay đề nghị UBND cấp xã xác minh nguồn gốc, tổ chức hòa giải và lập biên bản theo quy định để bảo vệ quyền sử dụng đất hợp pháp của gia đình tôi.
+[1]. Điều 138, 235, Luật 31/2024/QH15</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Câu trả lời đã trích dẫn Điều 138 và 235 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là các điều luật còn hiệu lực và phù hợp với tình huống tranh chấp đất đai và điều kiện cấp Giấy chứng nhận quyền sử dụng đất. Điều 138 quy định về điều kiện cấp Giấy chứng nhận cho người sử dụng đất không có giấy tờ, và Điều 235 quy định về thủ tục hòa giải tranh chấp đất đai. Các điều luật này đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết để giải quyết vấn đề của người hỏi.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="409.6" customHeight="1">
       <c r="A32" s="2" t="n">
@@ -1654,7 +1934,48 @@
 Có kết quả kg ak ( nhà bố mẹ e có 7 a c e ) nhưng mẫu đó kg có các thành viên ký ak</t>
         </is>
       </c>
-      <c r="C42" s="2" t="n"/>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Giấy tay bố mẹ viết, điểm chỉ và ký cho bạn thường chưa đủ để sang tên đất vì đất chưa có sổ và việc tặng cho chưa được đăng ký. Tuy nhiên, giấy này vẫn là chứng cứ quan trọng thể hiện ý chí của bố mẹ; phần quyền của bố có thể được xem là di sản và phải giải quyết cùng những người thừa kế của bố.
+Muốn tặng cho quyền sử dụng đất, thông thường người tặng phải có Giấy chứng nhận, đất không tranh chấp và còn thời hạn sử dụng. Đất chưa có sổ nên bố mẹ bạn chưa thể hoàn tất thủ tục tặng cho theo con đường thông thường. Điều 45 Luật Đất đai 2024
+Vì bố đã mất 2 năm:
+Nếu mảnh đất là tài sản chung của bố mẹ, trước hết xác định mẹ có 1/2; 1/2 của bố là di sản.
+Nếu bố không để lại di chúc hợp lệ, phần di sản này được chia cho mẹ, các con và cha/mẹ của bố (nếu còn sống vào thời điểm bố mất), theo hàng thừa kế thứ nhất. 7 anh chị em không ký giấy tay không làm giấy tự động vô hiệu, nhưng họ vẫn có quyền đối với phần di sản của bố nếu không có di chúc hợp pháp hoặc văn bản từ chối nhận di sản. Điều 651 Bộ luật Dân sự 2015
+Hướng làm an toàn:
+Làm thủ tục xin cấp Giấy chứng nhận lần đầu cho thửa đất, dựa vào việc bố mẹ đã ở ổn định hơn 30 năm; xin UBND cấp xã xác nhận nguồn gốc, thời điểm sử dụng, không tranh chấp.
+Đồng thời, các đồng thừa kế của bố lập văn bản khai nhận/thỏa thuận phân chia di sản tại tổ chức công chứng. Nếu mọi người đồng ý cho bạn hưởng phần của bố, cần ghi rõ thỏa thuận để bạn nhận phần đó.
+Mẹ ký hợp đồng tặng cho phần quyền của mẹ cho bạn; việc này thực hiện sau khi đủ điều kiện đăng ký/cấp sổ. Nếu một người thừa kế không đồng ý, có thể phát sinh tranh chấp và cần giải quyết tại Tòa án trước khi sang tên.
+Người đang sử dụng đất ổn định, không có giấy tờ vẫn có thể được xem xét cấp sổ tùy thời điểm sử dụng, việc không vi phạm pháp luật đất đai, không tranh chấp và điều kiện khác của từng trường hợp. Điều 138 Luật Đất đai 2024
+Bạn nên giữ bản gốc giấy tay, không tự ý sửa chữa; thu thập thêm giấy tờ về nhà đất, biên lai thuế, hộ khẩu cũ, điện nước, xác nhận hàng xóm và người làm chứng. Nếu giấy có nội dung rõ “cho toàn bộ đất/nhà cho bạn”, có chữ ký hoặc điểm chỉ của bố, mẹ và người làm chứng thì giá trị chứng minh sẽ tốt hơn, nhưng vẫn không thay thế thủ tục thừa kế và đăng ký đất đai.
+[1]. Điều 45, 138, Luật 31/2024/QH15
+[2]. Điều 651, Luật 91/2015/QH13</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Điều 45 và 138 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 651 của Bộ luật Dân sự 2015 (Luật số 91/2015/QH13). Tuy nhiên, không có nội dung cụ thể của các điều luật này được trích dẫn trong câu trả lời. Điều 45 và 138 của Luật Đất đai 2024 có thể liên quan đến việc cấp Giấy chứng nhận quyền sử dụng đất và các điều kiện liên quan, nhưng không được mô tả rõ ràng trong câu trả lời. Điều 651 của Bộ luật Dân sự 2015 liên quan đến thừa kế theo pháp luật, điều này đã được mô tả đúng trong câu trả lời. Tuy nhiên, việc không trích dẫn cụ thể nội dung điều luật và chỉ nêu số điều luật mà không có giải thích chi tiết làm giảm tính chính xác và đầy đủ của phần trích dẫn điều luật.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="409.6" customHeight="1">
       <c r="A43" s="2" t="n">
@@ -1752,7 +2073,44 @@
 Hiện tại sổ đỏ nhà em đang cắm khế vay ngân hàng nhưng em cần bản công chứng để làm hồ sơ du học nhưng giờ chỉ có bản photo và không có bản gốc nên đên ubnd xã họ không công chứng cho thì có các nào để công chứng không ạ. Mong mọi mng giải đáp giúp em ạ. Em cảm ơn</t>
         </is>
       </c>
-      <c r="C46" s="2" t="n"/>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: UBND xã không thể chứng thực bản sao sổ đỏ chỉ từ bản photocopy; bản sao chỉ được chứng thực khi xuất trình được bản chính để đối chiếu. Bạn nên xin ngân hàng cấp bản sao/giấy xác nhận có đóng dấu, hoặc đề nghị ngân hàng cho mượn bản gốc trong thời gian ngắn để đi chứng thực theo quy trình của họ.
+Người yêu cầu chứng thực bản sao phải xuất trình bản chính giấy tờ, văn bản làm căn cứ; người thực hiện chứng thực đối chiếu bản sao với bản chính rồi mới chứng thực. Vì vậy, chỉ mang bản photo thì UBND xã từ chối là đúng. Điều 20 Nghị định 23/2015/NĐ-CP
+Bạn liên hệ ngân hàng đang giữ sổ đỏ và đề nghị một trong các cách sau:
+Cấp bản sao Giấy chứng nhận từ hồ sơ tài sản bảo đảm, có xác nhận/đóng dấu của ngân hàng rằng bản sao được sao từ bản gốc ngân hàng đang lưu giữ;
+Cấp văn bản xác nhận ngân hàng đang giữ bản gốc sổ đỏ để bảo đảm khoản vay, kèm bản sao sổ đỏ đóng dấu giáp lai (nếu trường/đơn vị tiếp nhận hồ sơ du học chấp nhận);
+Đề nghị ngân hàng cho mượn bản gốc trong một buổi hoặc một ngày để bạn đem đi chứng thực. Thường ngân hàng sẽ yêu cầu giấy đề nghị, cam kết hoàn trả và có thể cử nhân viên đi cùng.
+Nếu đơn vị du học bắt buộc yêu cầu “certified true copy” do cơ quan nhà nước chứng thực, bạn cần hỏi rõ họ có chấp nhận bản sao do ngân hàng xác nhận hay không. Trường hợp không chấp nhận, cách thực tế nhất là làm việc với ngân hàng để xuất trình bản gốc tại UBND xã/phường hoặc tổ chức hành nghề công chứng để chứng thực, rồi trả lại ngay cho ngân hàng.
+Lưu ý: Công chứng/chứng thực bản sao không làm thay đổi tình trạng thế chấp; sổ đỏ vẫn đang bị đăng ký thế chấp và ngân hàng tiếp tục giữ bản gốc.
+[1]. Điều 20, Nghị định 23/2015/NĐ-CP</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Điều 20 của Nghị định 23/2015/NĐ-CP về chứng thực bản sao từ bản chính. Tuy nhiên, Nghị định này đã bị thay thế bởi Nghị định 101/2024/NĐ-CP, do đó, điều luật trích dẫn không còn hiệu lực. Câu trả lời đã bao phủ vấn đề về việc chứng thực bản sao khi không có bản gốc và các giải pháp làm việc với ngân hàng.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="176" customHeight="1">
       <c r="A47" s="2" t="n">
@@ -1764,7 +2122,60 @@
 P/s: vì 1 vài lý do nên em xin đăng ẩn danh</t>
         </is>
       </c>
-      <c r="C47" s="2" t="n"/>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Bạn có thể khởi kiện, nhưng khả năng yêu cầu Tòa “công nhận hợp đồng mua bán 100 m²” là thấp nếu chỉ mua bằng vi bằng, đất chưa tách thửa và bên bán chưa đủ điều kiện chuyển nhượng phần đất đó. Hướng thực tế thường là yêu cầu tuyên giao dịch vô hiệu, buộc bên bán hoàn trả toàn bộ tiền đã nhận, lãi/chênh lệch thiệt hại nếu chứng minh được, và xem xét lỗi của bên bán.
+Vi bằng chỉ ghi nhận sự kiện, hành vi mà Thừa phát lại trực tiếp chứng kiến (ví dụ giao tiền, giao giấy tờ); không thay thế hợp đồng chuyển nhượng quyền sử dụng đất đã được công chứng hoặc chứng thực. Vi bằng cũng không làm phát sinh quyền sử dụng đất riêng cho bạn.
+Để chuyển nhượng quyền sử dụng đất hợp pháp, bên bán phải có Giấy chứng nhận; đất không tranh chấp, không bị kê biên, còn thời hạn sử dụng và đáp ứng các điều kiện khác. Hợp đồng chuyển nhượng phải được công chứng hoặc chứng thực, trừ trường hợp luật có quy định riêng. Điều 45 Luật Đất đai 2024
+Trong trường hợp của bạn, việc chủ đất bán từng nền 100 m² khi:
+chưa tách thửa;
+chưa hoàn tất thủ tục hiến đất làm đường;
+chưa chuyển mục đích sang đất ở (nếu hiện chưa là đất ở);
+không thể cấp sổ riêng cho từng người mua;
+cho thấy đối tượng giao dịch có thể chưa đủ điều kiện để chuyển nhượng. Tòa khó có thể buộc cơ quan đất đai cấp sổ riêng nếu việc tách thửa không đáp ứng quy hoạch, diện tích tối thiểu hoặc điều kiện khác tại Đồng Nai.
+Bạn nên khởi kiện theo yêu cầu nào?
+Nên đặt yêu cầu chính là: tuyên hợp đồng/giấy mua bán đất vô hiệu; buộc bên bán hoàn trả số tiền đã nhận; bồi thường thiệt hại do lỗi làm giao dịch vô hiệu (nếu có). Khi giao dịch vô hiệu, các bên hoàn trả cho nhau những gì đã nhận; bên có lỗi gây thiệt hại phải bồi thường. Điều 131 Bộ luật Dân sự 2015
+Chỉ nên yêu cầu công nhận giao dịch và buộc tiếp tục thủ tục tách sổ nếu bạn có chứng cứ mạnh rằng:
+thửa đất đủ điều kiện tách thửa, phù hợp quy hoạch;
+bên bán có sổ và đã cam kết rõ thời hạn, nghĩa vụ tách sổ;
+trở ngại hiện nay chỉ là bên bán cố tình không thực hiện, không phải vướng quy định pháp luật;
+các bên có thể hoàn tất công chứng/chứng thực theo yêu cầu.
+Việc cần làm ngay:
+Thu thập vi bằng; giấy tay/hợp đồng đặt cọc hoặc mua bán; sao kê chuyển khoản, giấy giao nhận tiền; tin nhắn/quảng cáo về cam kết “hiến đường, tách sổ, lên thổ cư”; thông tin sổ gốc của chủ đất và hiện trạng quy hoạch.
+Gửi văn bản yêu cầu bên bán thực hiện cam kết trong thời hạn cụ thể, hoặc hoàn tiền. Đây là chứng cứ thể hiện bạn đã thiện chí giải quyết.
+Xin văn bản trả lời của UBND xã/cơ quan đăng ký đất đai về lý do không thể xây dựng, khả năng tách thửa, mục đích sử dụng đất, quy hoạch. Không chỉ dựa vào trao đổi miệng.
+Nếu không giải quyết, khởi kiện tại Tòa án nhân dân có thẩm quyền nơi có bất động sản. Với yêu cầu hoàn tiền, bạn có thể đề nghị Tòa áp dụng biện pháp khẩn cấp tạm thời nếu có căn cứ bên bán đang tẩu tán tài sản.
+Lưu ý về thời hiệu: yêu cầu Tòa tuyên giao dịch vô hiệu do vi phạm điều kiện về hình thức thường có thời hiệu 02 năm; nhưng cần xem chính xác nội dung giấy tờ, thời điểm các bên xác lập/thực hiện giao dịch và căn cứ vô hiệu để đánh giá. Điều 132 Bộ luật Dân sự 2015
+Bạn không nên tự xây dựng khi chưa có quyền sử dụng đất hợp pháp, chưa được cấp phép và chưa rõ quy hoạch. Việc xây dựng có thể phát sinh rủi ro bị xử lý hoặc khó đòi bồi thường về sau.
+[1]. Điều 45, Luật 31/2024/QH15
+[2]. Điều 131, 132, Luật 91/2015/QH13</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Câu trả lời đã trích dẫn Điều 45 của Luật Đất đai 2024 (Luật số 31/2024/QH15), điều này còn hiệu lực và phù hợp với vấn đề chuyển nhượng quyền sử dụng đất. Ngoài ra, câu trả lời cũng trích dẫn Điều 131 và 132 của Bộ luật Dân sự 2015 (Luật số 91/2015/QH13), các điều này cũng còn hiệu lực và liên quan đến việc tuyên bố giao dịch dân sự vô hiệu và thời hiệu khởi kiện. Các điều luật này đã bao phủ đầy đủ các khía cạnh pháp lý liên quan đến việc mua bán đất bằng vi bằng, điều kiện chuyển nhượng đất và khả năng khởi kiện để tuyên bố giao dịch vô hiệu.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="256" customHeight="1">
       <c r="A48" s="2" t="n">
@@ -1797,7 +2208,55 @@
 E cảm ơn ạ !</t>
         </is>
       </c>
-      <c r="C49" s="2" t="n"/>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Bố mẹ bạn có thể tặng cho đất cho 2 người con, nhưng nên đo đạc và xử lý chênh lệch 400 m² trước khi tách thửa/tặng cho. Phần 1.300 m² thực tế không tự động được công nhận toàn bộ; cần xác định phần tăng do sai số đo đạc hay do đất ven suối/lấn ra ngoài ranh giới sổ.
+1. Xử lý diện tích thực tế 1.300 m²
+Gia đình cần đề nghị Chi nhánh Văn phòng đăng ký đất đai đo đạc địa chính, xác định ranh giới, mốc giới và đối chiếu với hồ sơ cấp sổ năm 2004. Có hai khả năng:
+Nếu ranh giới sử dụng không thay đổi, không có tranh chấp và diện tích tăng là do sai số đo đạc/bản đồ cũ, gia đình có thể đề nghị cấp đổi sổ ghi theo diện tích đo thực tế. Phần đất ở tăng thêm có thể phải thực hiện nghĩa vụ tài chính, nhất là phần vượt hạn mức đất ở tại thời điểm cấp sổ cũ. Khoản 3 Điều 13 Nghị định 103/2024/NĐ-CP
+Nếu 400 m² tăng thêm là phần đất ven suối, đất công, đất thuộc hành lang bảo vệ nguồn nước hoặc diện tích gia đình sử dụng mở rộng ngoài ranh giới gốc, thì không thể tự động đưa vào sổ. Cơ quan đo đạc phải xác định chính xác hành lang suối, quy hoạch và nguồn gốc phần đất này trước.
+Lưu ý: Hai mặt giáp suối là yếu tố cần kiểm tra kỹ. Dù được sử dụng từ lâu, phần nằm trong hành lang bảo vệ nguồn nước hoặc đất do Nhà nước quản lý có thể bị hạn chế công nhận, xây dựng và tách thửa.
+2. Tách và tặng cho 2 con
+Sau khi có kết quả đo đạc, bố mẹ thực hiện theo thứ tự:
+Kiểm tra điều kiện tách thửa: đất có sổ, không tranh chấp, không bị kê biên, còn thời hạn sử dụng; hai thửa sau tách phải bảo đảm diện tích tối thiểu, kích thước cạnh và lối đi theo quy định của Hà Nội. Điều 220 Luật Đất đai 2024
+Lập hồ sơ tách thửa tại Chi nhánh Văn phòng đăng ký đất đai nơi có đất. Có thể đề nghị đo đạc/cấp đổi để điều chỉnh diện tích và tách thửa trong cùng quá trình nếu cơ quan đăng ký hướng dẫn.
+Sau khi có thửa mới, bố mẹ ký hợp đồng tặng cho quyền sử dụng đất cho từng người con tại tổ chức công chứng; sau đó nộp hồ sơ đăng ký biến động/sang tên.
+Điều kiện để bố mẹ tặng cho là đất có Giấy chứng nhận, không tranh chấp, không bị kê biên hoặc áp dụng biện pháp bảo đảm thi hành án, còn thời hạn sử dụng và không bị áp dụng biện pháp khẩn cấp tạm thời. Điều 45 Luật Đất đai 2024
+3. Về loại đất trên sổ
+Sổ ghi 250 m² đất ở sử dụng lâu dài và 650 m² đất vườn. Khi chia cho 2 con, không nên mặc định mỗi người được 125 m² đất ở; cần lập phương án tách sao cho cả hai thửa có phần đất ở, có lối đi hợp pháp và phù hợp quy hoạch. Phần đất vườn chỉ được chuyển sang đất ở khi được cơ quan có thẩm quyền cho phép và phải nộp tiền sử dụng đất theo quy định.
+Tặng cho giữa bố mẹ và con được miễn thuế thu nhập cá nhân và lệ phí trước bạ, nhưng vẫn có phí đo đạc, công chứng, cấp sổ và có thể có tiền sử dụng đất nếu đồng thời xin công nhận/chuyển mục đích phần đất ở tăng thêm. Điều 4 Luật Thuế thu nhập cá nhân 2007
+Hồ sơ nên chuẩn bị: sổ đỏ bản gốc; CCCD của bố mẹ và 2 con; giấy khai sinh chứng minh quan hệ cha mẹ-con; đăng ký kết hôn của bố mẹ; trích đo hiện trạng; hồ sơ cấp sổ năm 2004 nếu còn; giấy tờ chứng minh quá trình sử dụng ổn định phần diện tích tăng thêm.
+Bạn nên xin trước văn bản trả lời của cơ quan đăng ký đất đai về: phần 400 m² có thuộc hành lang suối/quy hoạch không, có được công nhận không, và điều kiện tách thửa áp dụng cho đúng vị trí đất tại Hà Nội.
+[1]. Điều 13, Nghị định 103/2024/NĐ-CP
+[2]. Điều 45, 220, Luật 31/2024/QH15
+[3]. Điều 4, Luật 04/2007/QH12</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Câu trả lời đã trích dẫn các điều luật từ Luật Đất đai 2024 và Nghị định 103/2024/NĐ-CP, là các văn bản còn hiệu lực hiện hành. Điều 13 Nghị định 103/2024/NĐ-CP liên quan đến việc xử lý diện tích đất tăng thêm do sai số đo đạc. Điều 45 và 220 Luật Đất đai 2024 quy định về điều kiện tặng cho và tách thửa đất. Điều 4 Luật Thuế thu nhập cá nhân 2007 quy định về miễn thuế thu nhập cá nhân trong trường hợp tặng cho giữa bố mẹ và con. Các điều luật này đã bao phủ đầy đủ các khía cạnh của câu hỏi, bao gồm xử lý diện tích đất tăng thêm, thủ tục tặng cho và các điều kiện liên quan.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="192" customHeight="1">
       <c r="A50" s="2" t="n">
@@ -1814,7 +2273,49 @@
 Em cảm ơn các bác</t>
         </is>
       </c>
-      <c r="C50" s="2" t="n"/>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Hai người con riêng của bố có thể có quyền hưởng thừa kế từ phần tài sản thuộc quyền của bố, nếu quan hệ cha-con được pháp luật xác định. Họ không có quyền đối với phần tài sản riêng của mẹ hoặc phần tài sản của mẹ trong khối tài sản chung vợ chồng; việc cùng/khác hộ khẩu không quyết định quyền sở hữu hay thừa kế.
+Nếu căn nhà, đất được tạo lập trong thời kỳ hôn nhân và không có căn cứ là tài sản riêng của mẹ, thường được coi là tài sản chung của bố mẹ, mỗi người có 1/2. Khi bố mất, bố chỉ được định đoạt bằng di chúc đối với 1/2 phần của bố, không thể cho ai phần của mẹ. Điều 33 Luật Hôn nhân và gia đình 2014 Điều 43 Luật Hôn nhân và gia đình 2014
+Bố có quyền lập di chúc để cho phần tài sản của mình cho bất kỳ ai, gồm 2 người con riêng. Nếu không có di chúc hợp pháp, di sản của bố sẽ chia theo pháp luật cho hàng thừa kế thứ nhất: mẹ bạn, toàn bộ các con của bố (gồm 3 anh em bạn và 2 con riêng), và cha mẹ của bố nếu còn sống tại thời điểm bố mất; mỗi người cùng hàng hưởng bằng nhau. Con sinh ngoài hôn nhân có quyền thừa kế ngang với con trong hôn nhân khi chứng minh được quan hệ cha-con. Điều 626 Bộ luật Dân sự 2015 Điều 651 Bộ luật Dân sự 2015
+Ví dụ: nhà là tài sản chung bố mẹ, bố mất không để lại di chúc, ông bà nội đã mất, có mẹ và 5 người con. Mẹ giữ 1/2 tài sản của mình; 1/2 của bố chia đều cho mẹ và 5 người con. Như vậy mẹ có 7/12 căn nhà, còn mỗi người con có 1/12.
+Để bảo vệ quyền lợi của mẹ và 3 anh em:
+Kiểm tra nguồn gốc nhà đất: tài sản có trước hôn nhân, được tặng cho riêng/thừa kế riêng của mẹ thì thuộc tài sản riêng của mẹ, bố và các con riêng không có quyền hưởng phần này.
+Lưu hồ sơ sổ đỏ, hợp đồng mua bán, giấy tờ tạo lập nhà đất, chứng từ tiền mua/xây nhà để xác định tỷ lệ sở hữu.
+Nếu bố còn sống và bố mẹ muốn ổn định tài sản, có thể lập văn bản thỏa thuận phân chia tài sản chung vợ chồng hoặc mẹ yêu cầu Tòa án chia tài sản chung trong thời kỳ hôn nhân khi có căn cứ; không được tự ý chuyển toàn bộ tài sản chung sang cho con nếu không có sự đồng ý hợp pháp của bố. Điều 38 Luật Hôn nhân và gia đình 2014
+Việc bố “bỏ đi”, có con với người khác trong khi chưa ly hôn không làm bố tự động mất quyền tài sản hoặc quyền lập di chúc. Nhưng nếu có hành vi vi phạm nghiêm trọng nghĩa vụ vợ chồng, mẹ bạn có thể cân nhắc thủ tục ly hôn, chia tài sản và yêu cầu giải quyết các quyền lợi liên quan.
+[1]. Điều 33, 38, 43, Luật 52/2014/QH13
+[2]. Điều 626, 651, Luật 91/2015/QH13</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Câu trả lời đã trích dẫn các điều luật liên quan đến quyền thừa kế và tài sản chung trong hôn nhân. Cụ thể:
+1. Điều 33, 38, 43 Luật Hôn nhân và gia đình 2014: Quy định về tài sản chung và riêng của vợ chồng, quyền yêu cầu chia tài sản chung trong thời kỳ hôn nhân.
+2. Điều 626, 651 Bộ luật Dân sự 2015: Quy định về quyền lập di chúc và thừa kế theo pháp luật.
+Các điều luật này đều còn hiệu lực và phù hợp với vấn đề pháp lý được hỏi, bao gồm quyền thừa kế của con riêng và quyền lập di chúc của bố.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="304" customHeight="1">
       <c r="A51" s="2" t="n">
@@ -1888,7 +2389,54 @@
 Tuy nhiên em vẫn chưa nhận được chuyển nhượng, chưa được bàn giao đủ đất (vẫn giữ nguyên hiện trạng) thì các nghĩa vụ này do bên nào chịu trách nhiệm ạ? Và mình cần làm gì để ép chủ cũ phải có trách nhiệm sớm đòi lại đất cho mình ạ</t>
         </is>
       </c>
-      <c r="C54" s="2" t="n"/>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Bên bán không thể viện lý do “đã công chứng hợp đồng” để phủi trách nhiệm giao đất đúng diện tích, ranh giới và trong tình trạng đủ điều kiện chuyển nhượng. Khi đất đang tranh chấp, hồ sơ sang tên không thể hoàn tất; bạn nên yêu cầu bên bán giải quyết tranh chấp trong thời hạn cụ thể hoặc thỏa thuận giảm giá/hoàn tiền, nếu không thì khởi kiện yêu cầu hủy/chấm dứt hợp đồng và hoàn trả tiền, bồi thường thiệt hại.
+Đất có tranh chấp thì không đủ điều kiện để thực hiện chuyển nhượng, trừ khi tranh chấp đã được giải quyết bằng quyết định/bản án có hiệu lực. Điều 45 Luật Đất đai 2024 Việc công chứng chỉ xác nhận hình thức, ý chí giao kết tại thời điểm ký; không bảo đảm thực tế đất không tranh chấp hoặc diện tích bàn giao đủ như hợp đồng.
+Về thuế và nghĩa vụ tài chính:
+Thuế thu nhập cá nhân từ chuyển nhượng về bản chất là nghĩa vụ của bên có thu nhập, tức bên bán. Hai bên có thể thỏa thuận bạn nộp thay, nhưng nếu giao dịch bị hủy/vô hiệu do bên bán không giao được đất đúng cam kết thì bạn có quyền yêu cầu bên bán hoàn lại khoản thuế bạn đã nộp thay và các chi phí hợp lý khác.
+Tiền sử dụng đất, thuế sử dụng đất phi nông nghiệp hằng năm trước ngày hoàn tất việc chuyển quyền/bàn giao thực tế thường cần đối chiếu điều khoản hợp đồng và nghĩa vụ gắn với người đứng tên, người sử dụng đất. Bạn chưa được đăng ký sang tên, chưa nhận đủ đất thì không nên tự nhận nghĩa vụ nộp các khoản còn tồn của bên bán nếu hợp đồng không quy định rất rõ.
+Thuế thu nhập từ chuyển nhượng bất động sản được xác định theo thời điểm bàn giao bất động sản; do đó, nếu chưa bàn giao được đầy đủ do tranh chấp, đây cũng là căn cứ để bạn yêu cầu làm rõ nghĩa vụ thuế và không tự nộp thêm khoản nào khi chưa có phương án xử lý. Điều 17 Nghị định 320/2025/NĐ-CP
+Bạn nên làm ngay:
+Yêu cầu cơ quan tiếp nhận hồ sơ cấp cho bạn văn bản/phiếu nêu rõ lý do chưa thể đăng ký sang tên, kết quả đo đạc và diện tích/rảnh giới đang tranh chấp. Xin trích đo địa chính, biên bản xác định mốc giới và thông tin thửa đất.
+Gửi văn bản cho bên bán, nêu rõ đất thiếu diện tích và đang tranh chấp nên không đủ điều kiện chuyển nhượng; yêu cầu họ chọn một trong hai phương án trong thời hạn 15–30 ngày:
+Hoàn tất việc giải quyết tranh chấp, bảo đảm bàn giao đủ diện tích đúng hợp đồng và đủ điều kiện sang tên; hoặc
+Ký phụ lục giảm giá, hoàn lại số tiền tương ứng diện tích thiếu và chi phí phát sinh; hoặc
+Hủy hợp đồng, hoàn lại tiền mua đất, tiền môi giới mà bên bán cam kết chịu (nếu có), chi phí công chứng, đo đạc, hồ sơ và thiệt hại thực tế.
+Không ký biên bản nhận bàn giao, xác nhận đã nhận đủ đất, phụ lục nhận giảm giá hoặc giấy cam kết tiếp tục mua nếu chưa có phương án rõ ràng. Không xây dựng, chuyển nhượng lại hoặc giao dịch tiếp đối với phần đất tranh chấp.
+Nếu hết thời hạn mà bên bán không giải quyết, khởi kiện tại Tòa án có thẩm quyền nơi có đất. Yêu cầu chính có thể là: buộc tiếp tục thực hiện hợp đồng và giao đất đủ điều kiện; hoặc hủy/chấm dứt hợp đồng, hoàn tiền và bồi thường. Bạn có thể đề nghị Tòa áp dụng biện pháp khẩn cấp tạm thời ngăn bên bán chuyển dịch tài sản nếu có dấu hiệu tẩu tán.
+Khi giao dịch dân sự vô hiệu, các bên phải hoàn trả cho nhau những gì đã nhận; bên có lỗi làm giao dịch vô hiệu phải bồi thường thiệt hại. Điều 131 Bộ luật Dân sự 2015
+Điểm quan trọng là xem đúng nội dung hợp đồng: diện tích ghi theo sổ hay theo thực đo; có ghi “chuyển nhượng toàn bộ thửa đất”, “theo hiện trạng”, “chênh lệch diện tích không điều chỉnh giá” hay không; thời hạn bàn giao; cam kết đất không tranh chấp; và điều khoản phạt vi phạm. Nếu hợp đồng chỉ bán theo diện tích trên sổ nhưng phần đất thực tế bị hàng xóm lấn khiến không thể đăng bộ, đây vẫn là rủi ro thuộc về bên bán khi họ cam kết đất đủ điều kiện chuyển nhượng.
+[1]. Điều 45, Luật 31/2024/QH15
+[2]. Điều 17, Nghị định 320/2025/NĐ-CP
+[3]. Điều 131, Luật 91/2015/QH13</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Điều 45 của Luật Đất đai 2024 và Điều 17 của Nghị định 320/2025/NĐ-CP, tuy nhiên, Nghị định 320/2025/NĐ-CP không tồn tại. Điều 131 của Bộ luật Dân sự 2015 được trích dẫn đúng và còn hiệu lực. Câu trả lời đã bao phủ phần lớn các vấn đề pháp lý liên quan đến tranh chấp đất đai và nghĩa vụ thuế, nhưng việc trích dẫn sai Nghị định làm giảm độ chính xác của phần trích dẫn điều luật.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="304" customHeight="1">
       <c r="A55" s="2" t="n">
@@ -2137,7 +2685,51 @@
 Chuyện là ba e có cho e 1 miếng đất và sắp tới e sẽ xây lại nhà trên đất này. Năm 1998 ba e có xây nhà trên đất này và đến 2007 ông bà e tách sổ đỏ riêng cho ba e. Đến 2013 có thay đổi để lên sổ hồng mới hay gì đó thì mẹ e hỏi bên xã ngta kêu nhà e khỏi đổi sổ hồng. Lúc đó e còn nhỏ và ba mẹ e nông dân cũng không biết nhiều nên để sổ đỏ cũ như năm 2007 luôn đến nay. Nay 2025 ba e sang tên cho e thì bắt buộc làm lại sổ hồng. Khi ra sổ rồi mới thấy là có dính quy hoạch kẻ vạch thẳng vào bản đồ đất luôn là gần 1 nửa diện tích đất. Loại đất trên sổ hồng hiện tại là Đất trồng cây lâu năm. E có thông tin từ bạn e là đất có cất nhà từ trước 2004 khi 2013 làm lại sổ sẽ được công nhận phần đất xây nhà là Đất Ở, nghĩa là cả thửa thì có phần xây nhà được tính thổ cư. Anh chị cho e hỏi thông tin này chính xác không và nếu thật vậy thì bây giờ e nên làm gì để được công nhận phần đất đó để đỡ tiền lên thổ cư cả thửa và khi quy hoạch sẽ được đền bù nhiều hơn. Nhà e xây giữa đất nên hiện tại 1 nửa dính quy hoạch và 1 nửa không dính. Và bây giờ nếu e đóng thổ cư e chỉ được đóng phần không dính quy hoạch. Nhưng phần quy hoạch có 1 nửa nhà e, nếu 2013 được công nhận phần đó thổ cư thì có phải sắp tới quy hoạch e được đền bù nhiều hơn, có giá hơn đất nông nghiệp đúng không ạ</t>
         </is>
       </c>
-      <c r="C65" s="2" t="n"/>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Thông tin bạn nghe là có cơ sở nhưng không tự động đúng. Nhà xây từ năm 1998 có thể là căn cứ để xin công nhận một phần diện tích là đất ở khi cấp đổi/cấp lại sổ, nhưng phải chứng minh thời điểm xây dựng, sử dụng ổn định và phải đối chiếu quy hoạch, nguồn gốc đất, hạn mức đất ở tại địa phương. Việc sổ hiện ghi toàn bộ là đất trồng cây lâu năm không làm bạn mất hẳn quyền đề nghị xem xét.
+Phần đất có nhà ở sử dụng ổn định từ năm 1998 thuộc giai đoạn từ 15/10/1993 đến trước 01/7/2014. Khi đủ điều kiện, diện tích đất ở có thể được xác định theo hạn mức giao đất ở tại địa phương; nếu diện tích nhà xây thực tế lớn hơn hạn mức thì có thể xem xét theo diện tích thực tế xây nhà. Điều 25 Nghị định 101/2024/NĐ-CP
+Tuy nhiên, trường hợp của bạn có điểm cần lưu ý: đất đã được cấp sổ cho bố từ năm 2007 và hiện vừa sang tên cho bạn, nên đây không đơn thuần là hồ sơ “cấp sổ lần đầu”. Bạn cần đề nghị cơ quan đăng ký đất đai kiểm tra lại hồ sơ cấp sổ năm 2007 và hồ sơ cấp đổi/sang tên gần đây: tại thời điểm đó, gia đình có kê khai nhà ở, hiện trạng nhà có được ghi nhận hay không, và vì sao toàn bộ thửa vẫn xác định là đất trồng cây lâu năm.
+Bạn nên thực hiện theo hướng sau:
+Nộp đơn tại Chi nhánh Văn phòng đăng ký đất đai nơi có đất, đề nghị:
+Sao lục hồ sơ địa chính, hồ sơ cấp sổ năm 2007;
+Xác minh hiện trạng, thời điểm xây dựng nhà từ năm 1998;
+Hướng dẫn thủ tục đăng ký biến động/cấp đổi để ghi nhận diện tích đất ở đối với phần có nhà ở;
+Trả lời bằng văn bản phần đất nào vướng quy hoạch, loại quy hoạch gì, đã có kế hoạch sử dụng đất hằng năm hoặc quyết định thu hồi đất chưa.
+Nộp kèm chứng cứ: giấy phép/xác nhận xây nhà cũ (nếu có), ảnh nhà qua các thời kỳ, biên lai điện nước lâu năm, hộ khẩu cũ, xác nhận của hàng xóm hoặc trưởng thôn/tổ dân phố, thuế nhà đất, hồ sơ cấp sổ năm 2007 và sổ mới.
+Không nên vội nộp tiền chuyển toàn bộ thửa sang đất ở. Trước hết hãy xác định diện tích nhà ở và sân, lối đi gắn liền với nhà có đủ cơ sở được công nhận là đất ở hay không. Chỉ khi không được công nhận mà bạn vẫn cần xây dựng thêm thì mới cân nhắc xin chuyển mục đích phần đất không vướng quy hoạch.
+Về quy hoạch: chỉ việc có đường kẻ quy hoạch trên sổ/bản đồ không đương nhiên làm mất quyền xin xác nhận nguồn gốc, hiện trạng nhà ở. Nhưng nếu đã có quyết định thu hồi đất hoặc kế hoạch sử dụng đất hằng năm cấp huyện trước đây xác định phải thu hồi, cơ quan có thể không cho chuyển mục đích sang đất ở đối với phần bị ảnh hưởng. Bạn cần kiểm tra bằng văn bản, không chỉ nghe thông tin miệng.
+Khi Nhà nước thu hồi, phần đất đủ điều kiện được công nhận quyền sử dụng đất có thể được bồi thường về đất. Với đất có nhà ở sử dụng ổn định trước 01/7/2014 thuộc trường hợp được xem xét cấp sổ, pháp luật có quy định bồi thường đất mà không bắt buộc phải đáp ứng điều kiện phù hợp quy hoạch; mức, diện tích được bồi thường còn phụ thuộc hồ sơ và hạn mức địa phương. Khoản 2 Điều 5 Nghị định 88/2024/NĐ-CP Điều 9 Nghị định 88/2024/NĐ-CP
+Vì vậy, mục tiêu đúng không phải là “đóng thổ cư để chắc được đền bù cao”, mà là làm rõ và bảo lưu chứng cứ rằng nhà đã tồn tại từ năm 1998, đề nghị công nhận đúng phần đất ở gắn với nhà. Nếu bị từ chối, yêu cầu cơ quan trả lời bằng văn bản nêu rõ căn cứ và loại quy hoạch đang áp dụng để xem xét khiếu nại.
+[1]. Điều 25, Nghị định 101/2024/NĐ-CP
+[2]. Điều 5, 9, Nghị định 88/2024/NĐ-CP</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Câu trả lời đã trích dẫn Điều 25 của Nghị định 101/2024/NĐ-CP và Điều 5, 9 của Nghị định 88/2024/NĐ-CP. Các điều luật này đều còn hiệu lực và liên quan đến việc công nhận đất ở và bồi thường khi thu hồi đất. Điều 25 của Nghị định 101/2024/NĐ-CP liên quan đến việc xác định diện tích đất ở khi có nhà xây dựng trước 01/7/2014. Điều 5 và 9 của Nghị định 88/2024/NĐ-CP liên quan đến bồi thường đất khi thu hồi. Các điều luật này đã bao phủ phần lớn câu hỏi về việc công nhận đất ở và bồi thường khi có quy hoạch, tuy nhiên, cần thêm thông tin cụ thể từ cơ quan chức năng để xác định chính xác trường hợp của người hỏi.</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="380" customHeight="1">
       <c r="A66" s="2" t="n">
@@ -2173,7 +2765,46 @@
 Xác định không bán / cắm ngân hàng</t>
         </is>
       </c>
-      <c r="C67" s="2" t="n"/>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Có khả năng sang tên được dù chủ cũ đã mất, nếu giấy viết tay mua bán đất năm 2000 có chứng thực hợp lệ của UBND xã và thể hiện rõ việc chuyển nhượng. Việc gia đình đang đóng thuế với tên mình là chứng cứ hỗ trợ, nhưng không tự thay thế thủ tục đăng ký sang tên.
+Bạn nên làm thủ tục sớm. Chưa sang tên thì trên pháp lý quyền sử dụng đất vẫn có thể đang đứng tên chủ cũ; về sau phát sinh tranh chấp với những người thừa kế của họ, thu hồi đất, cấp đổi sổ hoặc cần xác lập quyền cho con cháu sẽ phức tạp hơn, dù bạn không có ý định bán hay thế chấp.
+Hợp đồng chuyển nhượng quyền sử dụng đất phải được công chứng hoặc chứng thực, trừ trường hợp thuộc diện được pháp luật công nhận theo quy định chuyển tiếp. Giấy mua bán có dấu chứng thực của UBND xã tại thời điểm lập là yếu tố rất quan trọng; cần kiểm tra trên giấy có lời chứng thực, chữ ký/điểm chỉ của bên bán, thông tin thửa đất, giá/chuyển nhượng và chữ ký của các bên hay không. Điều 45 Luật Đất đai 2024
+Cách làm:
+Nộp hồ sơ đăng ký biến động/sang tên tại Bộ phận Một cửa hoặc Chi nhánh Văn phòng đăng ký đất đai nơi có đất.
+Hồ sơ nên có: sổ đỏ bản gốc; giấy mua bán viết tay bản gốc có xác nhận của xã; CCCD; tờ khai thuế, lệ phí trước bạ; biên lai thuế sử dụng đất các năm; giấy tờ chứng minh gia đình quản lý, sử dụng ổn định.
+Đề nghị cơ quan đăng ký đất đai kiểm tra hồ sơ lưu tại UBND xã về việc chứng thực hợp đồng năm 2000 nếu bản giấy có điểm chưa rõ.
+Việc toàn bộ vợ/chồng/con của chủ cũ đã mất không mặc nhiên làm giao dịch không thể sang tên. Nếu giao dịch đã hoàn thành từ năm 2000, bên bán đã ký và xã đã chứng thực thì quyền của họ về nguyên tắc đã chuyển giao; người thừa kế không thể tự lấy lý do người bán đã mất để phủ nhận giao dịch hợp pháp. Tuy nhiên, nếu giấy chỉ là “giấy viết tay có xác nhận chữ ký” hoặc nội dung không thể hiện rõ hợp đồng chuyển nhượng, cơ quan đăng ký có thể yêu cầu bổ sung hoặc từ chối; khi đó có thể phải khởi kiện yêu cầu Tòa án công nhận giao dịch/chuyển quyền sử dụng đất.
+Lưu ý thêm: nếu thửa đất là tài sản chung vợ chồng của chủ cũ mà chỉ một người ký giấy bán, cần xem có chữ ký/đồng ý của người còn lại hay không. Đây là điểm dễ phát sinh vướng mắc nhất.
+Bạn không nên nộp bản gốc giấy mua bán mà không có phiếu tiếp nhận hoặc bản sao chứng thực để lưu giữ. Nếu cơ quan từ chối, yêu cầu trả lời bằng văn bản, nêu rõ lý do và căn cứ pháp luật để có hướng khiếu nại hoặc khởi kiện.
+[1]. Điều 45, Luật 31/2024/QH15</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Câu trả lời có đề cập đến Điều 45 của Luật Đất đai 2024 (Luật số 31/2024/QH15), tuy nhiên không có nội dung cụ thể nào từ điều luật này được trích dẫn. Điều này làm cho việc đánh giá tính đúng đắn và hiệu lực của điều luật không thể thực hiện được. Ngoài ra, không có điều luật nào khác được trích dẫn để hỗ trợ cho các luận điểm trong câu trả lời. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="64" customHeight="1">
       <c r="A68" s="2" t="n">
@@ -2184,7 +2815,45 @@
           <t>Các bác cho e hỏi chút ạ. Đất đang bị tranh chấp, sổ đỏ cũng đã bị thu lại để cấp sổ mới và đang trong quá trình xử lí. Nhưng do bếp nhà e là mái ngói nên bị dột nát, vì thế e muốn sửa lại mái thay bằng mái tôn thì có được phép k ạ</t>
         </is>
       </c>
-      <c r="C68" s="2" t="n"/>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Bạn có thể sửa chữa để chống dột theo hướng giữ nguyên hiện trạng nhà, không cơi nới, không thay đổi kết cấu chịu lực, diện tích, chiều cao hoặc công năng. Tuy nhiên, vì đất đang tranh chấp và sổ đang bị thu hồi để xử lý, nên xin UBND xã/phường xác nhận hoặc hướng dẫn bằng văn bản trước khi làm để tránh bị cho là xây dựng mới/cơi nới.
+Việc thay mái ngói dột bằng mái tôn thường là sửa chữa, bảo trì nếu chỉ thay vật liệu mái trên khung/kết cấu hiện hữu. Công trình sửa chữa bên trong hoặc sửa chữa mặt ngoài không tiếp giáp đường đô thị có yêu cầu quản lý kiến trúc, không làm thay đổi công năng, không ảnh hưởng an toàn kết cấu chịu lực, phù hợp quy hoạch thì thuộc trường hợp được miễn giấy phép xây dựng. Khoản 2 Điều 89 Luật Xây dựng 2014
+Bạn không nên:
+Nâng mái, đổ cột/dầm mới, tăng chiều cao hoặc làm thêm tầng;
+Mở rộng bếp sang phần đất đang tranh chấp;
+Tháo dỡ toàn bộ rồi dựng lại như nhà mới;
+Xây cố định trên phần đất có ranh giới đang tranh chấp.
+Trước khi sửa, hãy chụp ảnh/video mái dột, hiện trạng bếp; lập danh mục hạng mục sửa chữa; thông báo bằng văn bản cho UBND xã/phường và bên đang tranh chấp rằng gia đình chỉ sửa mái để bảo đảm an toàn, không thay đổi hiện trạng, không làm phát sinh quyền đối với đất. Nếu địa phương yêu cầu hồ sơ hoặc giấy phép, đề nghị họ trả lời bằng văn bản.
+Sổ đang bị thu lại/cấp mới không đương nhiên cấm sửa chữa mái. Nhưng đất đang tranh chấp là lý do khiến việc xin giấy phép xây dựng mới rất khó, vì điều kiện cấp phép yêu cầu quyền sử dụng đất hợp pháp và hồ sơ đất đai phù hợp. Do đó, chỉ nên thực hiện mức độ sửa chữa tối thiểu để chống dột, an toàn sinh hoạt; không đầu tư xây dựng lớn cho đến khi tranh chấp và thủ tục sổ được giải quyết.
+[1]. Điều 89, Luật 50/2014/QH13</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Khoản 2 Điều 89 Luật Xây dựng 2014 (Luật số 50/2014/QH13) để giải thích về việc sửa chữa nhà mà không cần giấy phép xây dựng. Tuy nhiên, Luật Xây dựng 2014 đã bị thay thế bởi Luật Xây dựng 2020 (Luật số 62/2020/QH14), có hiệu lực từ 01/01/2021. Do đó, việc trích dẫn Luật Xây dựng 2014 là không còn hiệu lực. Câu trả lời đã bao phủ phần giải thích về việc sửa chữa nhà trong tình huống đất đang tranh chấp, nhưng sử dụng điều luật hết hiệu lực.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="224" customHeight="1">
       <c r="A69" s="2" t="n">
@@ -2199,7 +2868,49 @@
 Tôi chỉ nhớ là bà chị tôi có đưa tôi ký cái giấy gì đấy tại nhà mà do tui say xỉn với cận nặng quá nên không thấy chữ , vì tin chị nên tôi có ký . nhưng không ra công chứng mua bán sang tên gì cả.</t>
         </is>
       </c>
-      <c r="C69" s="2" t="n"/>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Đây là dấu hiệu rất nghiêm trọng. Bạn cần yêu cầu bảo vệ khẩn cấp tình trạng pháp lý của nhà đất, đồng thời tố giác nếu có dấu hiệu giả mạo/lừa ký giấy. Việc bạn từng ký một giấy tại nhà không đồng nghĩa bạn đã bán hoặc tặng cho nhà; chuyển nhượng nhà đất thông thường phải có hợp đồng công chứng/chứng thực và thủ tục đăng ký biến động.
+Bạn làm ngay các việc sau:
+Gửi đơn đề nghị ngăn chặn giao dịch đến Chi nhánh Văn phòng đăng ký đất đai nơi có nhà đất, nêu rõ: bạn là chủ cũ trên sổ, nghi việc sang tên không có ý chí tự nguyện hoặc có giả mạo, đang yêu cầu làm rõ. Kèm CCCD, bản sao sổ hồng cũ (nếu có), văn bản trả lời dữ liệu đất đai và các chứng cứ liên quan.
+Việc này nhằm hạn chế nguy cơ người đang đứng tên tiếp tục bán, tặng cho hoặc thế chấp.
+Yêu cầu cung cấp, sao lục hồ sơ biến động. Bạn là người có quyền, lợi ích trực tiếp bị ảnh hưởng nên cần đề nghị cơ quan đăng ký đất đai cho biết bằng văn bản: số hồ sơ sang tên, ngày đăng ký, căn cứ sang tên, tổ chức công chứng/chứng thực thực hiện, loại giao dịch (mua bán, tặng cho, thừa kế…), và bản sao tài liệu có chữ ký của bạn.
+Nếu họ từ chối nêu tên người đang đứng tên với lý do bảo mật, yêu cầu ban hành văn bản từ chối, ghi rõ căn cứ; đồng thời đề nghị cung cấp hồ sơ cho cơ quan công an hoặc Tòa án khi bạn tố giác/khởi kiện.
+Tố giác đến Công an cấp tỉnh/thành phố nơi có nhà đất hoặc Cơ quan Cảnh sát điều tra. Trong đơn, nêu rõ bạn phát hiện mình không còn đứng tên; nghi chữ ký/điểm chỉ bị giả mạo, hoặc bị lợi dụng khi say xỉn, mắt kém để ký giấy không được giải thích; đề nghị trưng cầu giám định chữ ký, chữ viết, dấu vân tay và xác minh hồ sơ công chứng.
+Không tự khẳng định chị bạn phạm tội nếu chưa có chứng cứ; chỉ trình bày sự việc và “đề nghị xác minh dấu hiệu”.
+Khởi kiện tại Tòa án nơi có nhà đất để yêu cầu tuyên giao dịch chuyển nhượng/tặng cho vô hiệu; hủy hoặc buộc thu hồi Giấy chứng nhận đã cấp, đăng ký biến động trái pháp luật; khôi phục quyền sử dụng đất cho bạn. Trong đơn có thể đề nghị Tòa áp dụng biện pháp khẩn cấp tạm thời: cấm chuyển dịch quyền về tài sản đối với nhà đất trong khi chờ giải quyết.
+Giấy chứng nhận đã cấp sai đối tượng, không đủ điều kiện cấp hoặc không đúng nguồn gốc có thể bị Nhà nước thu hồi; ngoài ra, Tòa án có thẩm quyền có thể tuyên hủy Giấy chứng nhận trong vụ án. Điều 152 Luật Đất đai 2024
+Nếu giao dịch được lập khi bạn không nhận thức, không làm chủ được hành vi; bị lừa dối; bị giả chữ ký; hoặc người ký không có quyền định đoạt, giao dịch có thể bị yêu cầu tuyên vô hiệu. Việc “không ra công chứng” là tình tiết có lợi cho bạn, nhưng vẫn phải kiểm tra vì có thể họ đã dùng hồ sơ công chứng/chứng thực mà bạn không biết.
+Bạn cần giữ và lập tức sao lưu: sổ hồng cũ; giấy tờ tùy thân; kết quả cung cấp dữ liệu đất đai; tin nhắn/cuộc gọi với chị; thông tin ngày, nơi, người chứng kiến việc bạn ký giấy; tài liệu chứng minh thời điểm đó bạn say xỉn hoặc thị lực kém. Đừng ký bất cứ giấy xác nhận, ủy quyền, thỏa thuận hoặc nhận tiền nào từ chị/người liên quan trước khi biết chính xác giao dịch nào đã được dùng để sang tên.
+Nếu nhà đất là tài sản chung vợ chồng, tài sản thừa kế hoặc có đồng sở hữu, cần đưa đầy đủ những người có quyền liên quan vào đơn tố giác và vụ kiện.
+[1]. Điều 152, Luật 31/2024/QH15</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Câu trả lời đã trích dẫn Điều 152 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều luật này liên quan đến việc thu hồi Giấy chứng nhận quyền sử dụng đất trong trường hợp cấp sai đối tượng, không đủ điều kiện cấp hoặc không đúng nguồn gốc. Điều luật này bao phủ phần yêu cầu hủy hoặc thu hồi Giấy chứng nhận đã cấp trái pháp luật. Tuy nhiên, câu trả lời chưa trích dẫn cụ thể các điều luật liên quan đến quy trình khởi kiện hoặc tố giác tại cơ quan công an, nhưng đã hướng dẫn chi tiết các bước cần thực hiện trong tình huống này.</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="409.6" customHeight="1">
       <c r="A70" s="2" t="n">
@@ -2260,7 +2971,56 @@
 Mình xin hỏi việc từ chối nhận hồ sơ cấp sổ đỏ lần đầu như vậy có đúng không, xin cảm ơn anh chị tư vấn và chia sẻ</t>
         </is>
       </c>
-      <c r="C72" s="2" t="n"/>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Bộ phận một cửa không nên chỉ trả hồ sơ với lý do biên nhận nộp tiền năm 1994 không có dấu, rồi bỏ qua toàn bộ căn cứ khác về nguồn gốc và quá trình sử dụng đất. Giấy biên nhận này có thể chưa đủ để tự nó chứng minh việc Nhà nước giao đất hợp pháp, nhưng gia đình vẫn có quyền yêu cầu cơ quan có thẩm quyền thụ lý, xác minh và xem xét cấp sổ theo diện đất đang sử dụng ổn định, không tranh chấp.
+Với thửa 223 m², cần tách hai vấn đề:
+Đơn xin cấp đất năm 1993 và biên nhận nộp 500.000 đồng không đóng dấu: đây là chứng cứ cần xác minh, nhưng khó được coi là quyết định giao đất hoặc giấy tờ giao đất hợp lệ nếu không xác định được người có thẩm quyền, hồ sơ xét giao đất và việc giao đất thực tế.
+Gia đình sử dụng liên tục, ranh giới rõ trong sổ mục kê, đóng thuế đất ở hằng năm đối với 200 m², đất không tranh chấp, phù hợp quy hoạch: đây là các chứng cứ độc lập quan trọng để xét cấp Giấy chứng nhận đối với đất không có giấy tờ. Điều 138 Luật Đất đai 2024
+Việc xã xác nhận không tranh chấp, phù hợp quy hoạch và có đường giao thông là thuận lợi, nhưng chưa phải quyết định công nhận quyền sử dụng đất. Cơ quan đăng ký đất đai vẫn cần xác minh thêm: thời điểm sử dụng thực tế, đất có phải quỹ đất công ích/đất công do xã quản lý không, việc “chuyển đổi đất phần trăm” năm nào, có vi phạm lấn chiếm hay giao đất trái thẩm quyền không.
+Bạn nên làm như sau:
+Nộp lại hồ sơ, kèm đơn đề nghị thụ lý và xác minh cấp sổ đối với cả hai thửa, trong đó đề nghị không đánh giá riêng biên nhận 1994 mà xem xét tổng thể quá trình sử dụng đất.
+Đề nghị UBND xã xác nhận bằng văn bản:
+Gia đình sử dụng thửa 223 m² từ thời điểm nào, liên tục và công khai;
+Đất có thuộc quỹ công ích, đất công hoặc đất do xã quản lý không;
+Căn cứ lập sổ mục kê, bản đồ 299 và việc gia đình đóng thuế đất ở 200 m²;
+Hồ sơ lưu về đơn xin đất, biên nhận nộp tiền, sổ thu/biên lai thu ngân sách năm 1993–1994.
+Kèm các tài liệu: sổ mục kê, trích đo, xác nhận không tranh chấp, biên lai thuế đất qua các năm, giấy tờ về nhà ở/cư trú, xác nhận của hộ liền kề, người làm chứng và bản gốc biên nhận 500.000 đồng.
+Nếu Bộ phận một cửa vẫn không nhận, yêu cầu họ lập phiếu từ chối tiếp nhận hồ sơ hoặc văn bản trả lời, ghi rõ lý do và căn cứ pháp luật. Không chấp nhận trả lời miệng.
+Điểm cần lưu ý: nếu thửa 223 m² được xác định là đất Nhà nước giao trái thẩm quyền sau ngày 01/7/2014 hoặc là đất công ích thì khả năng cấp sổ sẽ bị hạn chế. Ngược lại, nếu gia đình sử dụng ổn định từ trước 01/7/2014, không tranh chấp, không thuộc đất công và phù hợp điều kiện luật định, vẫn có cơ chế xem xét cấp Giấy chứng nhận dù không có giấy tờ hoàn chỉnh. Điều 138 Luật Đất đai 2024
+Nếu cơ quan tiếp nhận hoặc cơ quan có thẩm quyền ban hành văn bản từ chối không có căn cứ, bạn có thể khiếu nại đến người đứng đầu cơ quan đó hoặc khởi kiện hành chính. Quyền lựa chọn khiếu nại hoặc khởi kiện được pháp luật ghi nhận. Điều 7 Luật Khiếu nại 2011
+Bạn có thể viết ngắn trong đơn:
+Đề nghị cơ quan tiếp nhận, thụ lý và xác minh hồ sơ cấp Giấy chứng nhận đối với diện tích 223 m² theo quá trình sử dụng đất ổn định, công khai, không tranh chấp; đối chiếu sổ mục kê, hồ sơ 299, hồ sơ thu thuế và tài liệu lưu tại UBND xã. Biên nhận nộp tiền năm 1994 là tài liệu chứng minh bổ sung, không phải căn cứ duy nhất mà gia đình đề nghị xem xét.
+Do vị trí đất thuộc Hưng Yên, diện tích đất ở được công nhận và nghĩa vụ tài chính còn phụ thuộc hạn mức đất ở, quy định đang áp dụng của địa phương và kết quả xác minh nguồn gốc đất.
+[1]. Điều 138, Luật 31/2024/QH15
+[2]. Điều 7, Luật 02/2011/QH13</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Điều 138 Luật Đất đai 2024 và Điều 7 Luật Khiếu nại 2011. Tuy nhiên, không có nội dung cụ thể của các điều luật này được trích dẫn trong câu trả lời. Điều 138 Luật Đất đai 2024 có thể liên quan đến việc cấp Giấy chứng nhận quyền sử dụng đất, nhưng không có nội dung cụ thể nào được đưa ra để chứng minh điều này. Điều 7 Luật Khiếu nại 2011 liên quan đến quyền khiếu nại, nhưng cũng không có nội dung cụ thể nào được trích dẫn. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false do thiếu nội dung cụ thể và không có căn cứ rõ ràng từ các điều luật được trích dẫn.</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="304" customHeight="1">
       <c r="A73" s="2" t="n">
@@ -2296,7 +3056,47 @@
 Em xin cảm ơn ạ!</t>
         </is>
       </c>
-      <c r="C74" s="2" t="n"/>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Mẹ bạn vẫn có thể làm hồ sơ xin cấp sổ cho phần 40 m² còn lại, nhưng không thể khẳng định chắc chắn được cấp chỉ dựa vào giấy mua bán tay năm 2001. Cần xác minh nguồn gốc 100 m² của ông B/chú A, quá trình mẹ sử dụng ổn định 40 m², tình trạng tranh chấp và đặc biệt là diện tích 40 m² có đủ điều kiện tồn tại thành thửa riêng theo quy định nơi có đất hay không.
+Giấy mua bán 60 m² viết tay không có chứng thực không phải là hợp đồng chuyển nhượng hoàn chỉnh theo yêu cầu hình thức hiện nay. Tuy nhiên, đây vẫn là chứng cứ về việc nhận chuyển quyền và thời điểm sử dụng; cơ quan đất đai phải xem xét cùng các tài liệu khác như giấy mua bán có xác nhận phường giữa ông B và chú A, hiện trạng sử dụng, thuế, điện nước, nhà ở, xác nhận của hàng xóm và hồ sơ địa chính.
+Việc chú A và vợ đã mất không làm mẹ bạn mất quyền yêu cầu cấp sổ. Nhưng vì chú A là người đang đứng trong chuỗi giấy tờ, 3 người con của chú cần được mời xác minh/ý kiến khi UBND xã xác nhận nguồn gốc; nếu họ tranh chấp hoặc cho rằng 40 m² là di sản của chú A thì hồ sơ cấp sổ sẽ dừng để giải quyết tranh chấp.
+Mẹ bạn nên làm theo thứ tự:
+Đến UBND xã/phường và Chi nhánh Văn phòng đăng ký đất đai xin trích lục bản đồ, sổ mục kê, thông tin thửa đất 100 m² ban đầu: hiện ai kê khai/đứng tên, có thuộc đất công hay quy hoạch không, 100 m² đã được cấp sổ cho ai chưa.
+Nộp hồ sơ xin cấp Giấy chứng nhận lần đầu cho phần 40 m² đang sử dụng, kèm: giấy mua bán 60 m² bản gốc; bản photo giấy ông B bán cho chú A có xác nhận phường; giấy tờ về việc đã bán 30 m² cho cháu (nếu tìm lại được); giấy tờ nhà ở, điện nước, thuế; xác nhận ranh giới của các hộ liền kề; chứng cứ sử dụng liên tục từ năm 2001.
+Đề nghị UBND xã xác nhận bằng văn bản: thời điểm mẹ nhận đất, sử dụng ổn định/công khai, không tranh chấp, hiện trạng 40 m², nguồn gốc đất và việc đất có thuộc quỹ đất công hay không.
+Nếu 40 m² không đủ diện tích tối thiểu để tách thành thửa độc lập, vẫn cần đề nghị cơ quan đăng ký trả lời bằng văn bản hướng xử lý. Có nơi chỉ có thể cấp sổ khi thửa đất đã tồn tại trước thời điểm quy định hoặc phải hợp thửa với đất liền kề; không nên tự ý mua bán tiếp hay xây dựng trước khi rõ pháp lý.
+Người đang sử dụng đất không có giấy tờ vẫn có thể được xem xét cấp Giấy chứng nhận nếu sử dụng ổn định, không vi phạm pháp luật đất đai, không tranh chấp và đáp ứng điều kiện của từng trường hợp. Điều 138 Luật Đất đai 2024
+Bạn cần đặc biệt kiểm tra giấy tờ về 30 m² đã bán cho cháu. Nếu giấy năm 2001 ghi mẹ mua toàn bộ 60 m², còn hiện mẹ chỉ quản lý 40 m², hồ sơ cần thể hiện rõ phần 30 m² đã chuyển cho ai, vị trí/rang giới thế nào để tránh bị chồng lấn hoặc bị coi là không xác định được thửa đất.
+Nếu cơ quan từ chối nhận hoặc từ chối cấp sổ, yêu cầu họ trả lời bằng văn bản, ghi rõ lý do và căn cứ pháp luật. Khi đó mới đánh giá được có nên khiếu nại hay cần khởi kiện để xác định quyền sử dụng đất.
+[1]. Điều 138, Luật 31/2024/QH15</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Câu trả lời có trích dẫn Điều 138 của Luật Đất đai 2024 (Luật số 31/2024/QH15), tuy nhiên không có nội dung cụ thể của điều luật này được nêu ra trong câu trả lời. Điều này làm cho việc đánh giá tính đúng đắn và hiệu lực của điều luật trở nên khó khăn. Ngoài ra, câu trả lời không trích dẫn các điều luật cụ thể liên quan đến việc cấp Giấy chứng nhận quyền sử dụng đất trong trường hợp không có giấy tờ hợp lệ, điều này có thể làm giảm mức độ bao phủ của câu trả lời đối với vấn đề pháp lý được hỏi.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="409.6" customHeight="1">
       <c r="A75" s="2" t="n">
@@ -2360,7 +3160,52 @@
 Xin hỏi loại đất này có làm đuoc sổ đỏ k? Cần những giấy tờ gì ạ</t>
         </is>
       </c>
-      <c r="C77" s="2" t="n"/>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Có thể làm sổ đỏ lần đầu. Bằng khoán điền thổ là giấy tờ rất có giá trị để chứng minh nguồn gốc đất; giấy mua bán tay năm 1979 cũng có thể được xem xét nếu UBND cấp xã xác nhận đất đã được sử dụng trước ngày 15/10/1993. Tuy nhiên, vì ông bà đã mất, người cháu đang ở chỉ được đứng tên sổ nếu là người thừa kế hợp pháp hoặc có sự thống nhất của các đồng thừa kế.
+Bằng khoán điền thổ do chế độ cũ cấp thuộc nhóm giấy tờ về quyền sử dụng đất. Người đang sử dụng đất ổn định có loại giấy này có thể được cấp Giấy chứng nhận và thường không phải nộp tiền sử dụng đất, nếu đất không có tranh chấp và không thuộc trường hợp bị loại trừ. Điều 137 Luật Đất đai 2024
+Giấy mua bán viết tay từ năm 1979 cũng là chứng cứ quan trọng. Nếu UBND cấp xã xác nhận việc mua bán và sử dụng đất đã có từ trước ngày 15/10/1993, đây là căn cứ để xem xét cấp sổ. Điều 137 Luật Đất đai 2024
+Điểm cần giải quyết trước là thừa kế:
+Nếu ông bà không có di chúc cho riêng người cháu, mảnh đất là di sản của ông bà. Hàng thừa kế thứ nhất gồm các con của ông bà, vợ/chồng còn sống tại thời điểm người mất, cha mẹ của người mất nếu còn. Cháu chỉ hưởng trực tiếp nếu cha/mẹ của cháu đã mất trước hoặc cùng thời điểm với ông/bà, hoặc có di chúc, hoặc các đồng thừa kế thỏa thuận cho cháu nhận đất. Điều 651 Bộ luật Dân sự 2015
+Việc cháu trông coi, sinh sống tại đất không tự động làm cháu là chủ sử dụng duy nhất.
+Hồ sơ nên chuẩn bị:
+Bằng khoán điền thổ bản gốc; giấy mua bán tay năm 1979 bản gốc;
+Giấy chứng tử của ông bà; giấy khai sinh, giấy tờ chứng minh quan hệ các con/cháu;
+Di chúc (nếu có), hoặc văn bản khai nhận/thỏa thuận phân chia di sản có công chứng;
+CCCD người đề nghị cấp sổ;
+Giấy tờ chứng minh sử dụng ổn định: biên lai thuế, hộ khẩu/cư trú cũ, điện nước, ảnh nhà, xác nhận hàng xóm;
+Đơn đăng ký, cấp Giấy chứng nhận lần đầu và trích đo địa chính theo hướng dẫn nơi có đất.
+Nếu các con của ông bà đều thống nhất để cháu nhận đất, cách thuận lợi nhất là lập văn bản thỏa thuận phân chia di sản tại tổ chức công chứng, ghi rõ giao toàn bộ quyền sử dụng đất cho cháu. Sau đó nộp cùng hồ sơ cấp sổ tại Bộ phận Một cửa hoặc Chi nhánh Văn phòng đăng ký đất đai nơi có đất.
+Nếu có người thừa kế không đồng ý, hoặc tranh chấp nguồn gốc/diện tích đất, cơ quan đất đai sẽ không cấp sổ cho riêng cháu cho đến khi tranh chấp được giải quyết.
+[1]. Điều 137, Luật 31/2024/QH15
+[2]. Điều 651, Luật 91/2015/QH13</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Câu trả lời đã trích dẫn Điều 137 của Luật Đất đai 2024, điều này liên quan đến việc cấp Giấy chứng nhận quyền sử dụng đất cho các trường hợp có giấy tờ về quyền sử dụng đất từ chế độ cũ, như Bằng khoán điền thổ. Điều này còn hiệu lực và phù hợp với tình huống. Ngoài ra, Điều 651 Bộ luật Dân sự 2015 cũng được trích dẫn đúng để giải thích về quyền thừa kế, điều này cũng còn hiệu lực và phù hợp với tình huống thừa kế đất đai. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết cho việc cấp sổ đỏ và thừa kế.</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="288" customHeight="1">
       <c r="A78" s="2" t="n">
@@ -2587,7 +3432,49 @@
 E xin cam on ạ</t>
         </is>
       </c>
-      <c r="C88" s="2" t="n"/>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Để chắc chắn mảnh đất thuộc về con 12 tuổi và hạn chế tranh chấp, hai vợ chồng nên làm hợp đồng tặng cho quyền sử dụng đất cho con tại tổ chức công chứng, rồi đăng ký sang tên cho con. Chỉ viết giấy “để lại sau này cho con” không đủ an toàn vì có thể bị thay đổi, hủy bỏ hoặc tranh chấp.
+Vì đất đang đứng tên cả hai vợ chồng, cả hai phải cùng ký hợp đồng tặng cho. Việc định đoạt bất động sản là tài sản chung vợ chồng cần có sự thỏa thuận bằng văn bản của cả hai. Điều 35 Luật Hôn nhân và gia đình 2014
+Người dưới 18 tuổi vẫn có thể nhận tặng cho quyền sử dụng đất. Do con 12 tuổi chưa đủ năng lực tự mình xác lập giao dịch, cha/mẹ sẽ đại diện ký, nhưng cần tránh xung đột lợi ích: cả cha và mẹ nên thống nhất việc tặng cho, và đề nghị công chứng viên hướng dẫn cách thể hiện người đại diện cho con theo đúng hồ sơ. Điều 21 Bộ luật Dân sự 2015
+Sau công chứng, nộp hồ sơ đăng ký biến động tại Bộ phận Một cửa hoặc Chi nhánh Văn phòng đăng ký đất đai nơi có đất. Hợp đồng tặng cho chỉ có hiệu lực đối với quyền sử dụng đất sau khi được đăng ký theo quy định. Điều 45 Luật Đất đai 2024
+Hồ sơ thường gồm: sổ đỏ/sổ hồng bản gốc; CCCD của vợ chồng; giấy đăng ký kết hôn; giấy khai sinh của con; hợp đồng tặng cho đã công chứng; tờ khai thuế, lệ phí trước bạ. Tặng cho giữa cha mẹ và con được miễn thuế thu nhập cá nhân và lệ phí trước bạ, nhưng vẫn có phí công chứng, đo đạc/cấp sổ nếu phát sinh. Điều 4 Luật Thuế thu nhập cá nhân 2007
+Lưu ý: Sau khi sang tên cho con, về nguyên tắc cha mẹ không thể tự bán, thế chấp hay tặng cho lại đất của con. Việc định đoạt bất động sản của người chưa thành niên phải vì lợi ích của con và tuân thủ điều kiện đại diện theo pháp luật; vì vậy hãy cân nhắc kỹ trước khi sang tên toàn bộ.
+[1]. Điều 35, Luật 52/2014/QH13
+[2]. Điều 21, Luật 91/2015/QH13
+[3]. Điều 45, Luật 31/2024/QH15
+[4]. Điều 4, Luật 04/2007/QH12</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>1. Điều 35 Luật Hôn nhân và gia đình 2014: Quy định về việc định đoạt tài sản chung của vợ chồng, cần có sự thỏa thuận của cả hai. Luật này còn hiệu lực.
+2. Điều 21 Bộ luật Dân sự 2015: Quy định về năng lực hành vi dân sự của người chưa thành niên, người đại diện theo pháp luật. Luật này còn hiệu lực.
+3. Điều 45 Luật Đất đai 2024: Quy định về hiệu lực của hợp đồng tặng cho quyền sử dụng đất sau khi đăng ký. Luật này còn hiệu lực.
+4. Điều 4 Luật Thuế thu nhập cá nhân 2007: Quy định về miễn thuế thu nhập cá nhân cho tặng cho giữa cha mẹ và con. Luật này còn hiệu lực.
+Các điều luật trích dẫn đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết cho việc tặng cho quyền sử dụng đất cho con chưa thành niên, bao gồm cả thủ tục và miễn thuế.</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="350" customHeight="1">
       <c r="A89" s="2" t="n">
@@ -2620,7 +3507,49 @@
 Xin tư vấn trình tự đi giúp em ah.</t>
         </is>
       </c>
-      <c r="C90" s="2" t="n"/>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Bạn chưa nên vội nhận mình “hủy mua” và chấp nhận mất cọc. Nếu kết quả đo đạc cho thấy thửa đất sai tọa độ, lấn sang đất hàng xóm nên không thể sang tên đúng hiện trạng, bên bán có dấu hiệu không bảo đảm điều kiện chuyển nhượng và không thể giao đất đúng cam kết; bạn có cơ sở yêu cầu hoàn lại cọc, thậm chí phạt cọc nếu chứng minh lỗi thuộc bên bán.
+Đất chuyển nhượng phải có Giấy chứng nhận, không tranh chấp và đáp ứng điều kiện giao dịch. Việc hai đội đo độc lập cùng xác định có lấn ranh là chứng cứ rất quan trọng cho thấy hiện trạng/hồ sơ thửa đất có vấn đề. Điều 45 Luật Đất đai 2024
+Trình tự nên làm:
+Lấy văn bản của đơn vị đo đạc: trích đo, sơ đồ chồng lấn, biên bản xác định mốc ranh; yêu cầu cơ quan đăng ký đất đai hoặc bộ phận tiếp nhận hồ sơ ghi rõ lý do chưa thể sang tên.
+Gửi thông báo bằng văn bản cho bên bán, không dùng cụm “em hủy mua”. Nêu rằng: đất có sai lệch tọa độ/lấn ranh theo kết quả đo ngày…; không đủ điều kiện hoàn tất sang tên; yêu cầu bên bán trong 7–15 ngày:
+khắc phục, giải quyết ranh giới và bảo đảm sang tên được đúng diện tích; hoặc
+chấm dứt hợp đồng đặt cọc, hoàn lại tiền cọc; nếu bên bán có lỗi thì thực hiện mức phạt cọc theo thỏa thuận.
+Không ký giấy “tự nguyện bỏ cọc”, “hủy cọc do bên mua đổi ý”, hoặc biên bản xác nhận bên bán không sai. Những giấy này sẽ rất bất lợi khi tranh chấp.
+Nếu bên bán không trả tiền, khởi kiện tại Tòa án nơi bị đơn cư trú hoặc, nếu tranh chấp gắn trực tiếp với quyền sử dụng thửa đất, tại Tòa án nơi có đất. Yêu cầu Tòa tuyên chấm dứt/hủy hợp đồng đặt cọc do lỗi bên bán, buộc hoàn cọc và phạt cọc/bồi thường theo hợp đồng.
+Theo quy định về đặt cọc, nếu bên nhận đặt cọc từ chối giao kết hoặc thực hiện hợp đồng thì phải trả lại tiền cọc và một khoản tương đương tiền cọc, trừ khi hai bên có thỏa thuận khác. Ngược lại, nếu Tòa xác định bạn đơn phương không mua vì lý do cá nhân thì bên bán có thể được giữ cọc. Điều 328 Bộ luật Dân sự 2015
+Việc bên bán nói bạn “vu khống” không làm mất quyền yêu cầu kiểm tra hiện trạng đất. Bạn chỉ nên trình bày đúng sự thật theo tài liệu: “kết quả đo đạc thể hiện có chồng lấn/sai lệch ranh”, không khẳng định họ cố ý lừa đảo khi chưa có kết luận.
+Bạn cần giữ: hợp đồng đặt cọc; chứng từ chuyển cọc; tin nhắn về diện tích, ranh giới, cam kết sang tên; hai kết quả đo; ảnh mốc ranh; giấy hẹn hoặc văn bản cơ quan đất đai. Điểm quyết định là điều khoản cọc ghi thế nào: bên bán có cam kết đất “không tranh chấp”, “đủ điều kiện sang tên”, “đúng diện tích/sổ” hay không.
+[1]. Điều 45, Luật 31/2024/QH15
+[2]. Điều 328, Luật 91/2015/QH13</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Điều 45 của Luật Đất đai 2024 và Điều 328 của Bộ luật Dân sự 2015. Tuy nhiên, không có nội dung cụ thể nào từ Điều 45 của Luật Đất đai 2024 được trích dẫn hoặc giải thích rõ ràng trong câu trả lời. Điều 328 của Bộ luật Dân sự 2015 liên quan đến quy định về đặt cọc, nhưng không có nội dung cụ thể nào từ điều này được trích dẫn hoặc giải thích rõ ràng trong câu trả lời. Do đó, mặc dù các điều luật được đề cập có thể tồn tại và còn hiệu lực, nhưng việc trích dẫn không rõ ràng và không đầy đủ nội dung cụ thể từ các điều luật này khiến tiêu chí trích dẫn điều luật bị đánh giá là không đạt.</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="409.6" customHeight="1">
       <c r="A91" s="2" t="n">
@@ -2657,7 +3586,46 @@
 Em cám ơn các bác nhiều lắm ạ</t>
         </is>
       </c>
-      <c r="C92" s="2" t="n"/>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Lý do “đất có nguồn gốc Nhà nước giao đất có thu tiền sử dụng đất nên không được tách” là không phù hợp với Điều 220 Luật Đất đai 2024. Điều luật này không cấm tách thửa chỉ vì nguồn gốc đất như bạn nêu; cần kiểm tra các điều kiện thực tế và quy định diện tích tối thiểu tại Phú Thọ.
+Với đất ở 180 m², dự kiến tách thành 2 thửa 5 m × 18 m = 90 m²/thửa:
+Nếu là đất ở đô thị, mỗi thửa đạt tối thiểu 50 m², mặt tiền tối thiểu 3,5 m, chiều sâu tối thiểu 4 m;
+Nếu là đất ở nông thôn, mỗi thửa đạt tối thiểu 80 m², mặt tiền tối thiểu 4 m, chiều sâu tối thiểu 5 m.
+Như vậy, về diện tích và kích thước bạn nêu thì mỗi thửa 90 m², ngang 5 m, sâu 18 m đều đạt. Điều 11 Quyết định 116/2025/QĐ-UBND
+Điều kiện chung còn phải bảo đảm: thửa đất đã có sổ; còn thời hạn sử dụng; không tranh chấp, không bị kê biên hoặc áp dụng biện pháp khẩn cấp tạm thời; hai thửa sau tách có lối đi và kết nối với đường giao thông công cộng. Điều 220 không đặt điều kiện cấm tách đối với trường hợp nhận chuyển nhượng đất mà nguồn gốc ban đầu là Nhà nước giao đất có thu tiền sử dụng đất. Điều 220 Luật Đất đai 2024
+Bạn nên yêu cầu Văn phòng đăng ký đất đai trả lời bằng văn bản: họ cho rằng bạn “vi phạm khoản/điểm nào Điều 220”, và lý do cụ thể là gì. Không nên chỉ nhận câu trả lời miệng.
+Sau đó, nộp hồ sơ tách thửa gồm đơn đăng ký biến động/tách thửa, sổ đỏ bản gốc, CCCD và trích đo địa chính theo hướng dẫn. Nếu VPĐKĐĐ ra văn bản từ chối mà vẫn lấy lý do nguồn gốc giao đất có thu tiền, bạn có thể khiếu nại người đứng đầu cơ quan đã từ chối; hoặc khởi kiện hành chính khi cho rằng hành vi từ chối là trái luật. Điều 7 Luật Khiếu nại 2011
+Lưu ý: Nếu trên sổ có ghi hạn chế quyền sử dụng đất, đang thế chấp, có quy hoạch/dự án đã có quyết định thu hồi, hoặc phần đường đi sau tách không bảo đảm thì đó có thể là lý do hợp pháp khác. Bạn cần yêu cầu họ chỉ rõ đúng lý do này, không chấp nhận cách giải thích chung chung.
+[1]. Điều 220, Luật 31/2024/QH15
+[2]. Điều 7, Luật 02/2011/QH13</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Câu trả lời có trích dẫn Điều 220 của Luật Đất đai 2024, tuy nhiên không có nội dung cụ thể của điều luật này để xác định tính chính xác và hiệu lực. Ngoài ra, câu trả lời cũng đề cập đến Điều 7 của Luật Khiếu nại 2011, điều này là đúng và còn hiệu lực. Tuy nhiên, không có trích dẫn cụ thể từ Luật Đất đai 2024 để xác định rõ ràng việc tách thửa có bị cấm hay không dựa trên nguồn gốc đất. Cần có thêm thông tin chi tiết về quy định của Luật Đất đai 2024 và các văn bản hướng dẫn liên quan để đánh giá đầy đủ.</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="256" customHeight="1">
       <c r="A93" s="2" t="n">
@@ -2713,7 +3681,42 @@
 Hiện tại giáp danh nhà e vs hàng xóm đang có 1 khoảng 20-30 cm không thuộc về ai. Bên địa chính nói đất của nhà nc vậy thì em muốn mua chỗ đất đó để gộp vs sổ nhà em thì thủ tục như thế nào ạ</t>
         </is>
       </c>
-      <c r="C95" s="2" t="n"/>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Bạn không thể “mua ngay” 20–30 cm đất đó chỉ theo thỏa thuận với địa chính. Nếu đúng là đất do Nhà nước quản lý và là phần đất nhỏ hẹp xen kẹt, gia đình có thể làm đơn đề nghị Nhà nước giao đất có thu tiền để hợp thửa với đất nhà mình; nhưng phải qua xác minh, công khai và quyết định của cơ quan có thẩm quyền.
+Trước hết, đề nghị UBND xã/phường hoặc Chi nhánh Văn phòng đăng ký đất đai đo đạc, xác định rõ: phần đó thuộc thửa đất nào, có thực sự là đất công/đất Nhà nước quản lý không, có nằm trong hành lang giao thông, thủy lợi, mương thoát nước hay quy hoạch công trình công cộng không. Không nên tự rào, sử dụng hoặc xây dựng lên phần đất này.
+Phần đất nhỏ hẹp, xen kẹt có thể được giao cho người sử dụng đất liền kề nếu: không đủ diện tích tách thửa độc lập; phù hợp quy hoạch; không thuộc khu vực có dự án/công trình đã xác định; không tranh chấp; và không cần dùng vào mục đích công cộng. Việc giao đất phải ưu tiên mục đích công cộng; chỉ khi không sử dụng vào mục đích công cộng mới xem xét giao có thu tiền hoặc cho thuê cho hộ liền kề. Điều 47 Nghị định 102/2024/NĐ-CP
+Bạn nộp đơn đề nghị giao đất có thu tiền sử dụng đất đối với diện tích nhỏ hẹp xen kẹt để hợp thửa tại Bộ phận Một cửa UBND xã/phường nơi có đất. Trong đơn ghi vị trí, diện tích ước tính, giáp ranh, nhu cầu hợp thửa; đề nghị xác minh nguồn gốc, đưa vào danh mục đất nhỏ hẹp xen kẹt và công khai lấy ý kiến.
+Nếu được chấp thuận, bạn phải nộp tiền sử dụng đất theo thông báo; sau đó đo đạc và làm thủ tục hợp thửa với thửa đất nhà mình. Nếu hàng xóm cũng có nhu cầu, cơ quan có thẩm quyền sẽ xem xét quy hoạch và điều kiện thực tế, không mặc nhiên giao toàn bộ cho một bên. Điều 47 Nghị định 102/2024/NĐ-CP
+Vì bạn chưa cho biết tỉnh/thành nơi có đất, chưa thể xác định quy trình, cơ quan giải quyết và đơn giá cụ thể của địa phương.
+[1]. Điều 47, Nghị định 102/2024/NĐ-CP</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Câu trả lời đã trích dẫn Điều 47 Nghị định 102/2024/NĐ-CP, quy định về việc giao đất nhỏ hẹp xen kẹt cho người sử dụng đất liền kề. Nghị định này còn hiệu lực và phù hợp với tình huống hỏi về việc mua phần đất nhỏ hẹp không thuộc về ai để gộp vào sổ đỏ. Điều luật đã bao phủ phần chính của câu hỏi về thủ tục và điều kiện để có thể hợp thửa phần đất này.</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="409.6" customHeight="1">
       <c r="A96" s="2" t="n">
@@ -2749,7 +3752,46 @@
 Sổ thì tên mẹ e nhưng trong thời kỳ hôn nhân</t>
         </is>
       </c>
-      <c r="C97" s="2" t="n"/>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Em trai bạn không thể “từ chối nhận di sản từ mẹ” khi mẹ vẫn còn sống; chưa có di sản thừa kế để từ chối. Vì đất được tạo lập trong thời kỳ hôn nhân, dù sổ chỉ đứng tên mẹ thì thường vẫn là tài sản chung của bố mẹ; mẹ không thể tự tặng cho toàn bộ thửa đất khi bố chỉ đang biệt tích.
+Sổ chỉ đứng tên mẹ không mặc nhiên là tài sản riêng của mẹ. Tài sản có được trong thời kỳ hôn nhân thường là tài sản chung, trừ khi chứng minh được mẹ được tặng cho riêng, thừa kế riêng, mua bằng tài sản riêng hoặc có thỏa thuận khác. Quyền sử dụng đất là tài sản chung có thể chỉ ghi tên một người trên sổ nếu vợ chồng có thỏa thuận đứng tên đại diện. Điều 33 Luật Hôn nhân và gia đình 2014 Khoản 4 Điều 135 Luật Đất đai 2024
+Việc tặng cho toàn bộ đất là định đoạt bất động sản chung, cần có sự thỏa thuận bằng văn bản của cả bố và mẹ. Bố “đi biệt tích” không đồng nghĩa bố đã mất hoặc mất quyền đối với 1/2 tài sản. Điều 35 Luật Hôn nhân và gia đình 2014
+Hướng xử lý:
+Nếu đất là tài sản riêng của mẹ: mẹ có thể tặng cho bạn; em trai không cần làm giấy từ chối di sản.
+Nếu là tài sản chung: mẹ chỉ có thể tặng cho phần quyền của mẹ; muốn tặng toàn bộ cần có chữ ký/ủy quyền hợp lệ của bố, hoặc mẹ cần yêu cầu Tòa án giải quyết tình trạng bố vắng mặt, quản lý tài sản và/hoặc chia tài sản chung theo thủ tục phù hợp. Không nên làm “giấy từ chối di sản” tại xã vì giấy này không giải quyết được quyền của bố.
+Nếu bố đã biệt tích liên tục từ 02 năm trở lên, không có tin tức xác thực dù đã áp dụng đầy đủ biện pháp thông báo, mẹ hoặc người có quyền lợi liên quan có thể yêu cầu Tòa án tuyên bố bố mất tích. Sau đó mới xem xét việc quản lý, định đoạt tài sản theo quyết định của Tòa; tuyên bố mất tích không tự động chuyển phần đất của bố thành đất riêng của mẹ. Điều 68 Bộ luật Dân sự 2015
+Khi làm thủ tục, cần kiểm tra nguồn gốc thửa đất, thời điểm mua/cấp sổ, giấy đăng ký kết hôn và thời gian bố bỏ đi để chọn đúng phương án.
+[1]. Điều 33, 35, Luật 52/2014/QH13
+[2]. Điều 135, Luật 31/2024/QH15
+[3]. Điều 68, Luật 91/2015/QH13</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Điều 33 và 35 của Luật Hôn nhân và gia đình 2014, và Điều 68 của Bộ luật Dân sự 2015, đều còn hiệu lực và đúng với tình huống về tài sản chung và biệt tích. Tuy nhiên, câu trả lời trích dẫn Điều 135 của Luật Đất đai 2024, nhưng không có nội dung cụ thể của điều luật này trong câu trả lời, và không rõ ràng về tính hiệu lực của điều luật này trong bối cảnh câu hỏi. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false.</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="409.6" customHeight="1">
       <c r="A98" s="2" t="n">
@@ -2843,7 +3885,47 @@
 Vậy hỏi: khi được cấp sổ đỏ lần đầu thì trong trường hợp này có cần đóng tiền sử dụng đất hay là không ạ?</t>
         </is>
       </c>
-      <c r="C101" s="2" t="n"/>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Không thể khẳng định “không phải nộp tiền sử dụng đất” chỉ vì đất khai phá, sử dụng trước năm 1980. Với thông tin bạn nêu là không có giấy tờ và hiện không có nhà, phần đất đang thể hiện là ONT + CLN sẽ được xem xét riêng: phần được công nhận là đất ở có thể phải nộp tiền sử dụng đất; phần được công nhận là đất trồng cây lâu năm thì không nộp tiền sử dụng đất.
+Đất không có giấy tờ vẫn có thể được xem xét cấp sổ nếu gia đình sử dụng ổn định trước ngày 01/7/2014, không vi phạm pháp luật đất đai, không tranh chấp và được UBND cấp xã xác nhận các điều kiện theo luật. Điều 138 Luật Đất đai 2024
+Vì trên đất không có nhà, không nên mặc định toàn bộ hoặc một phần thửa đất được công nhận là đất ở chỉ do bản đồ ghi “ONT + CLN”. Cần xác minh: diện tích ONT trên bản đồ là bao nhiêu; việc ghi ONT dựa vào hồ sơ nào; gia đình có từng có nhà, nền nhà, công trình phục vụ đời sống hay không; đất có thuộc đất công ích, đất do Nhà nước quản lý hoặc lấn chiếm không.
+Nếu cơ quan có thẩm quyền công nhận một phần là đất ở cho người sử dụng đất không có giấy tờ, đất sử dụng trước 18/12/1980 thì mức thu tiền sử dụng đất hiện hành về nguyên tắc là:
+Trong hạn mức công nhận đất ở: 10% giá đất;
+Vượt hạn mức công nhận đất ở: 30% giá đất;
+Nếu được công nhận là đất phi nông nghiệp khác: 40% giá đất.
+Điều 11 Nghị định 103/2024/NĐ-CP
+Phần được công nhận là đất trồng cây lâu năm (CLN) không phát sinh tiền sử dụng đất khi cấp sổ; nhưng có thể có lệ phí cấp sổ, phí đo đạc, trích lục hồ sơ theo mức của địa phương.
+Bạn nên nộp hồ sơ xin cấp sổ lần đầu và đề nghị UBND xã xác nhận bằng văn bản: thời điểm khai phá/sử dụng trước năm 1980, sử dụng liên tục, không tranh chấp, nguồn gốc đất, không thuộc đất công. Đồng thời yêu cầu cơ quan đăng ký đất đai xác định rõ diện tích nào được công nhận ONT và diện tích nào là CLN trước khi ban hành thông báo nghĩa vụ tài chính.
+[1]. Điều 138, Luật 31/2024/QH15
+[2]. Điều 11, Nghị định 103/2024/NĐ-CP</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Câu trả lời đã trích dẫn Điều 138 của Luật Đất đai 2024 và Điều 11 của Nghị định 103/2024/NĐ-CP. Cả hai văn bản này đều còn hiệu lực và phù hợp với tình huống cấp sổ đỏ lần đầu cho đất sử dụng trước năm 1980. Điều 138 Luật Đất đai 2024 quy định về điều kiện cấp sổ đỏ cho đất không có giấy tờ nhưng sử dụng ổn định, không tranh chấp. Điều 11 Nghị định 103/2024/NĐ-CP quy định về mức thu tiền sử dụng đất khi công nhận đất ở trong hạn mức và vượt hạn mức. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý liên quan đến việc cấp sổ đỏ và nghĩa vụ tài chính.</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="128" customHeight="1">
       <c r="A102" s="2" t="n">
@@ -2858,7 +3940,45 @@
 Em xin cảm ơn.</t>
         </is>
       </c>
-      <c r="C102" s="2" t="n"/>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Bạn được phép dành một phần đất làm lối đi để tách thửa; phần lối đi phải kết nối với đường giao thông công cộng. Luật không ấn định chung lối đi phải rộng bao nhiêu mét, nên 3 m có thể được chấp nhận nhưng còn phải đáp ứng quy định tách thửa và yêu cầu hạ tầng hiện hành của Đồng Nai.
+Khi tách thửa, thửa đất phía sau phải có lối đi hợp lý, kết nối với đường giao thông công cộng, bảo đảm cấp nước và thoát nước. Nếu bạn dành một phần thửa đất ở hoặc thửa có đất ở để làm lối đi thì không phải chuyển mục đích sử dụng đất đối với phần lối đi đó. Điều 220 Luật Đất đai 2024
+Với đất ngang 8 m, dài 138 m, nếu chừa 3 m làm đường thì phần đất còn lại phía trước/sau chỉ còn ngang khoảng 5 m. Bạn cần kiểm tra đồng thời:
+Mỗi thửa sau tách có đủ diện tích, kích thước cạnh tối thiểu theo quy định Đồng Nai;
+Phần 3 m đường được thể hiện rõ trên trích đo và có kết nối trực tiếp đường công cộng;
+Có phương án thoát nước, không vướng quy hoạch/hành lang bảo vệ công trình;
+Thửa đất không tranh chấp, không bị ngăn chặn giao dịch.
+Bạn nên nộp đơn đề nghị cung cấp thông tin/quy hoạch và hướng dẫn tách thửa tại Bộ phận Một cửa xã Lộc Ninh hoặc Chi nhánh Văn phòng đăng ký đất đai nơi có đất, kèm sơ đồ dự kiến tách 8 m × 138 m và phần đường 3 m. Yêu cầu trả lời bằng văn bản về: bề rộng lối đi tối thiểu, số thửa được tách, diện tích/kích thước mỗi thửa sau tách và việc phần đường có phải hiến cho Nhà nước hay chỉ là lối đi chung.
+Không nên tự gọi là “hiến đất” trước khi được hướng dẫn. Nếu hiến hẳn cho Nhà nước làm đường, cần thủ tục tiếp nhận và cập nhật đất công; còn nếu chỉ phục vụ các thửa phía sau, có thể thiết lập lối đi chung và ghi nhận rõ quyền sử dụng, quản lý phần đường trong hồ sơ tách thửa.
+[1]. Điều 220, Luật 31/2024/QH15</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Điều 220 của Luật Đất đai 2024 (Luật số 31/2024/QH15), tuy nhiên không có nội dung cụ thể của điều luật này trong câu trả lời. Điều này làm cho việc xác định tính đúng đắn và hiệu lực của điều luật không thể thực hiện được. Câu trả lời đã bao phủ phần lớn các yếu tố cần thiết để tách thửa, nhưng không có điều luật cụ thể nào được trích dẫn để hỗ trợ cho các yêu cầu về diện tích tối thiểu, kích thước cạnh tối thiểu, và các yêu cầu khác liên quan đến quy hoạch và hạ tầng.</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="409.6" customHeight="1">
       <c r="A103" s="2" t="n">
@@ -2892,7 +4012,43 @@
 T11/2024 e có lấy ck .Tháng 2025 bố e có cho e 1 mảnh đất đứng riêng e . Theo hình thức cho tặng. Mn cho e hỏi bây giờ e muốn bán hay thế chấp ở ngân hàng thi có liên quan j đến ck ko ạ và có cần chữ kí ko ạ . E cảm ơn ạ</t>
         </is>
       </c>
-      <c r="C104" s="2" t="n"/>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Nếu mảnh đất được bố tặng cho riêng bạn, hợp đồng tặng cho và sổ hồng chỉ ghi tên bạn, thì đây là tài sản riêng; bạn có thể bán hoặc thế chấp mà không cần chồng ký. Nếu văn bản tặng cho không ghi cho riêng, hoặc đã nhập tài sản này vào khối tài sản chung, chồng có thể có quyền liên quan.
+Tài sản được vợ hoặc chồng được tặng cho riêng trong thời kỳ hôn nhân là tài sản riêng của người đó. Người có tài sản riêng có quyền tự mình chiếm hữu, sử dụng, định đoạt tài sản riêng; vì vậy chồng không cần ký hợp đồng bán hoặc thế chấp. Điều 43 Luật Hôn nhân và gia đình 2014 Điều 44 Luật Hôn nhân và gia đình 2014
+Bạn nên kiểm tra 3 điểm trước khi giao dịch:
+Hợp đồng tặng cho ghi rõ: “tặng cho riêng bà …”; không ghi tặng cho “vợ chồng” hoặc ghi chung cả hai.
+Sổ hồng cấp sau tặng cho chỉ ghi tên bạn.
+Không có văn bản thỏa thuận nhập thửa đất vào tài sản chung vợ chồng.
+Khi công chứng bán/thế chấp, mang theo sổ hồng, hợp đồng tặng cho, CCCD và giấy đăng ký kết hôn. Công chứng viên thường yêu cầu các giấy tờ này để xác định đây là tài sản riêng. Nếu hồ sơ không thể hiện rõ là “tặng cho riêng”, nên làm văn bản xác nhận tài sản riêng hoặc văn bản thỏa thuận chế độ tài sản vợ chồng có công chứng trước khi bán/thế chấp để tránh bị yêu cầu chữ ký của chồng.
+[1]. Điều 43, 44, Luật 52/2014/QH13</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Điều 43 và 44 của Luật Hôn nhân và gia đình 2014 (Luật số 52/2014/QH13), quy định về tài sản riêng của vợ, chồng. Tuy nhiên, các điều luật này vẫn còn hiệu lực và đúng với tình huống hỏi về tài sản riêng trong hôn nhân. Tuy nhiên, câu trả lời không trích dẫn điều luật nào từ Luật Đất đai 2024 hoặc các nghị định mới liên quan đến việc chuyển nhượng hoặc thế chấp quyền sử dụng đất, do đó không đáp ứng đầy đủ tiêu chí trích dẫn điều luật.</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="409.6" customHeight="1">
       <c r="A105" s="2" t="n">
@@ -2954,7 +4110,46 @@
 đất mua 2002 mình có cất căn nhà tiền chế năm 2024 nay làm sổ lần đầu phòng kinh tế hạ tầng khảo sát có nhà và trả hồ sơ không cấp sổ vậy có phải tháo gỡ không</t>
         </is>
       </c>
-      <c r="C107" s="2" t="n"/>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Chưa thể kết luận bạn phải tháo dỡ nhà tiền chế chỉ vì cơ quan khảo sát thấy có nhà và trả hồ sơ cấp sổ. Việc cấp Giấy chứng nhận quyền sử dụng đất lần đầu phải xét riêng nguồn gốc, quá trình sử dụng đất; còn căn nhà xây năm 2024 có thể không được chứng nhận quyền sở hữu nếu xây dựng không hợp pháp, nhưng không đương nhiên làm mất quyền xin cấp sổ đất.
+Cơ quan tiếp nhận phải trả lời bằng văn bản, ghi rõ lý do, căn cứ pháp luật và nội dung cần bổ sung/khắc phục. Bạn nên yêu cầu “phiếu từ chối tiếp nhận/giải quyết hồ sơ” hoặc văn bản trả hồ sơ; không nên tự tháo dỡ khi chưa biết lý do chính thức.
+Điều cần kiểm tra là nhà tiền chế có vi phạm hay không: xây trên đất nông nghiệp, đất không phù hợp quy hoạch/mục đích sử dụng; thuộc khu vực phải có giấy phép xây dựng nhưng không có phép; hoặc lấn ranh, hành lang bảo vệ công trình. Nếu có quyết định xử phạt kèm biện pháp buộc tháo dỡ của cơ quan có thẩm quyền thì mới phải chấp hành việc tháo dỡ theo quyết định đó. Việc xây công trình không đúng mục đích sử dụng đất có thể là hành vi bị cấm và bị xử lý. Điều 3 Luật Đất đai 2024 Điều 9 Luật Đất đai 2024
+Đất mua từ năm 2002 vẫn có thể được xem xét cấp sổ nếu sử dụng ổn định, không tranh chấp và đáp ứng điều kiện theo từng loại giấy tờ/nguồn gốc đất. Nhà xây sau này là tài sản gắn liền với đất; việc ghi nhận nhà trên sổ cần có hồ sơ chứng minh việc tạo lập hợp pháp, không phải cứ có nhà là hồ sơ đất bị bác. Luật Đất đai 2024
+Bạn nên làm ngay:
+Nộp/yêu cầu văn bản trả hồ sơ, hỏi rõ họ từ chối cấp sổ đất hay chỉ chưa ghi nhận quyền sở hữu nhà.
+Chuẩn bị giấy mua bán năm 2002, giấy tờ giao đất/chuyển nhượng (nếu có), biên lai thuế, xác nhận sử dụng ổn định, giấy xác nhận không tranh chấp và hồ sơ hiện trạng.
+Nếu lý do là nhà xây không phép, đề nghị cơ quan hướng dẫn bằng văn bản phương án xử lý; có thể tách yêu cầu cấp sổ đất trước, chưa đề nghị chứng nhận căn nhà.
+Nếu văn bản từ chối không có căn cứ hoặc áp dụng sai luật, bạn có quyền khiếu nại đến người đứng đầu cơ quan đã trả hồ sơ hoặc khởi kiện hành chính.
+Vì bạn chưa nêu tỉnh/thành phố và lý do ghi trên giấy trả hồ sơ, chưa thể xác định chính xác có phải tháo dỡ hay không. Bạn có thể chụp/chép nguyên văn lý do trả hồ sơ và cho biết đất là đất ở hay đất nông nghiệp, ở tỉnh nào; tôi sẽ đối chiếu cụ thể.
+[1]. Điều 3, 9, Luật 31/2024/QH15</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Câu trả lời có trích dẫn Điều 3 và Điều 9 của Luật Đất đai 2024 (Luật số 31/2024/QH15). Tuy nhiên, không có nội dung cụ thể nào từ các điều luật này được nêu ra trong câu trả lời, và việc trích dẫn này không rõ ràng, không cung cấp thông tin cụ thể về nội dung điều luật liên quan đến vấn đề cấp sổ đỏ và việc xây dựng nhà trên đất. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là không đạt yêu cầu.</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="409.6" customHeight="1">
       <c r="A108" s="2" t="n">
@@ -3015,7 +4210,47 @@
 Em xin cảm ơn</t>
         </is>
       </c>
-      <c r="C110" s="2" t="n"/>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Cách ít chi phí và gọn nhất thường là chú tặng cho bố bạn trước, rồi bố tặng cho bạn. Tuy nhiên, cách này phải làm 2 lần thủ tục; đổi lại, cả hai lần tặng cho giữa anh em ruột và giữa cha-con đều thuộc diện miễn thuế thu nhập cá nhân, miễn lệ phí trước bạ nếu chứng minh được quan hệ.
+Không nên để chú tặng thẳng cho bạn nếu mục tiêu là tiết kiệm: quan hệ chú–cháu không thuộc diện miễn thuế. Khi đó, người nhận có thể phải nộp thuế thu nhập cá nhân 10% trên phần giá trị quà tặng vượt 20 triệu đồng; đồng thời có thể phát sinh lệ phí trước bạ. Điều 61 Nghị định 253/2026/NĐ-CP Điều 67 Thông tư 89/2026/TT-BTC
+Cách thực hiện:
+Chú và bố lập hợp đồng tặng cho quyền sử dụng đất tại tổ chức công chứng. Vì là anh/em ruột, cần giấy khai sinh hoặc giấy tờ hộ tịch chứng minh cùng cha hoặc mẹ.
+Nộp hồ sơ đăng ký sang tên cho bố tại cơ quan đăng ký đất đai cấp tỉnh/xã theo nơi có đất; đề nghị miễn thuế, lệ phí kèm giấy tờ chứng minh quan hệ.
+Sau khi sổ đã đứng tên bố, bố và bạn lập hợp đồng tặng cho; tiếp tục làm thủ tục sang tên và hồ sơ miễn thuế, lệ phí vì là cha–con.
+Chỉ tặng cho đúng phần diện tích được phép tách thửa. Nếu “cắt đất” là một phần thửa đất đang đứng tên chú, phải kiểm tra điều kiện tách thửa tại địa phương trước; có thể làm hồ sơ tách thửa đồng thời với tặng cho.
+Điều kiện cơ bản để chú được tặng cho là đất có Giấy chứng nhận, không tranh chấp, không bị kê biên/áp dụng biện pháp bảo đảm thi hành án và còn thời hạn sử dụng đất. Điều 45 Luật Đất đai 2024
+Lưu ý quan trọng: dù ông bà nội là nguồn gốc đất, hiện sổ đã mang tên chú thì về thủ tục trước mắt chú là người có quyền định đoạt. Nhưng nếu sổ được cấp sai nguồn gốc, còn tranh chấp di sản của ông bà, hoặc các đồng thừa kế chưa thống nhất, cần xử lý thừa kế trước khi tặng cho để tránh tranh chấp và nguy cơ bị hủy giao dịch sau này.
+[1]. Điều 61, Nghị định 253/2026/NĐ-CP
+[2]. Điều 67, Thông tư 89/2026/TT-BTC
+[3]. Điều 45, Luật 31/2024/QH15</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Điều 61 Nghị định 253/2026/NĐ-CP, Điều 67 Thông tư 89/2026/TT-BTC và Điều 45 Luật Đất đai 2024. Tuy nhiên, các văn bản này không tồn tại hoặc không có hiệu lực tại thời điểm hiện tại (2023). Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false. Câu trả lời đã bao phủ các bước thực hiện thủ tục tặng cho đất giữa các thành viên gia đình và các lưu ý về thuế, lệ phí, nhưng không có điều luật cụ thể nào được trích dẫn đúng và còn hiệu lực để hỗ trợ cho các bước này.</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="409.6" customHeight="1">
       <c r="A111" s="2" t="n">
@@ -3057,7 +4292,45 @@
 vậy khi ly hôn em có cần giấy tờ gì để chứng minh đó là tài sản riêng của em nữa không ạ. và nhà ở là tài sản chung thì xử lý như nào</t>
         </is>
       </c>
-      <c r="C112" s="2" t="n"/>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Đất của bạn có cơ sở mạnh để được xác định là tài sản riêng vì được mẹ tặng cho riêng trong thời kỳ hôn nhân và sổ chỉ đứng tên bạn. Tuy nhiên, khi ly hôn bạn vẫn nên xuất trình hồ sơ tặng cho để chứng minh rõ đây là tặng cho riêng, bởi nếu không chứng minh được thì tài sản tranh chấp có thể bị coi là tài sản chung.
+Bạn cần lưu giữ và nộp cho Tòa án khi có tranh chấp:
+Hợp đồng/văn bản tặng cho, trong đó thể hiện mẹ tặng cho riêng bạn;
+Sổ hồng bản gốc hoặc bản sao chứng thực, thể hiện nguồn gốc “nhận tặng cho từ hộ bà…” và chỉ tên bạn;
+Hồ sơ sang tên/cấp sổ tại cơ quan đăng ký đất đai, biên lai nghĩa vụ tài chính;
+Nếu người tặng là “hộ bà xxx”, cần thêm giấy tờ chứng minh các thành viên hộ gia đình có quyền sử dụng đất đã đồng ý việc tặng cho riêng bạn.
+Tài sản được tặng cho riêng trong thời kỳ hôn nhân là tài sản riêng; quyền sử dụng đất có sau kết hôn cũng không là tài sản chung nếu được tặng cho riêng. Ngược lại, khi không có chứng cứ chứng minh là tài sản riêng thì pháp luật suy đoán đó là tài sản chung. Điều 43 Luật Hôn nhân và gia đình 2014 Điều 33 Luật Hôn nhân và gia đình 2014
+Về căn nhà: nếu xây trong thời kỳ hôn nhân bằng tiền/thu nhập chung hoặc hai vợ chồng cùng tạo lập, nhà thường là tài sản chung dù đất là của riêng bạn. Khi ly hôn, thông thường giá trị đất riêng vẫn thuộc bạn; phần giá trị căn nhà được chia theo công sức đóng góp, hoàn cảnh và các yếu tố khác. Nếu không thể chia nhà bằng hiện vật, người tiếp tục sở hữu đất và nhà có thể nhận nhà, rồi thanh toán lại cho người kia phần giá trị họ được hưởng.
+Bạn nên thu thập thêm chứng cứ về tiền xây nhà: hợp đồng xây dựng, hóa đơn vật liệu, sao kê chuyển khoản, giấy vay tiền, người làm chứng. Nếu bạn chứng minh nhà được xây hoàn toàn từ tiền riêng của mình (ví dụ tiền được tặng cho riêng, thừa kế riêng, hoặc tài sản riêng có trước hôn nhân) thì có thể yêu cầu xác định cả nhà là tài sản riêng; còn nếu chồng có đóng góp tiền, công sức hoặc cải tạo đáng kể thì họ có thể yêu cầu chia giá trị phần đóng góp.
+[1]. Điều 33, 43, Luật 52/2014/QH13</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Điều 33 và 43 của Luật Hôn nhân và gia đình 2014 (Luật số 52/2014/QH13), tuy nhiên không có điều luật nào từ Luật Đất đai 2024 hoặc các nghị định mới liên quan đến việc xác định tài sản riêng hay chung trong trường hợp này. Luật Hôn nhân và gia đình 2014 vẫn còn hiệu lực và đúng đắn trong việc xác định tài sản riêng và chung trong hôn nhân. Tuy nhiên, câu trả lời không trích dẫn điều luật từ Luật Đất đai 2024, điều này có thể cần thiết để xác định rõ hơn về quyền sử dụng đất và tài sản gắn liền với đất.</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="365" customHeight="1">
       <c r="A113" s="2" t="n">
@@ -3095,7 +4368,46 @@
 Mong các anh/chị chia sẻ cách hiểu và áp dụng thực tế. Em cảm ơn ạ.</t>
         </is>
       </c>
-      <c r="C114" s="2" t="n"/>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Kết luận: Không. Hợp rồi tách thửa không làm phần đất trồng cây lâu năm của thửa 2 tự phát sinh thành đất ở nếu gia đình không được cơ quan có thẩm quyền cho phép chuyển mục đích sử dụng đất. Khi tách lại, diện tích đất ở chỉ được xác định trong phạm vi diện tích đất ở hợp pháp đã có của thửa 1.
+Cần lưu ý, nội dung bạn nêu về Nghị quyết 254/2025/QH15 có thể đang hiểu chưa chính xác: Điều 4 của Nghị quyết này không quy định việc hợp thửa được miễn điều kiện cùng mục đích sử dụng đất. Điều 4 Nghị quyết 254/2025/QH15
+Theo Luật Đất đai, về nguyên tắc hợp thửa phải cùng mục đích sử dụng đất. Riêng trường hợp hợp toàn bộ hoặc một phần thửa có đất ở và đất khác trong cùng thửa với nhau, hoặc với thửa đất ở, được áp dụng ngoại lệ. Nếu các thửa khác nhau về mục đích sử dụng thì phải đồng thời làm thủ tục chuyển mục đích để thống nhất mục đích sử dụng. Điều 220 Luật Đất đai 2024
+Áp vào trường hợp của gia đình:
+Thửa 1 sau khi hợp vẫn có cơ cấu: một phần đất ở và một phần đất trồng cây lâu năm;
+Thửa 2 cũng chỉ là đất trồng cây lâu năm;
+Khi tách lại, có thể bố trí một thửa nhận phần đất ở vốn có của thửa 1; phần đất tách từ khu vực thửa 2 ban đầu vẫn là đất trồng cây lâu năm.
+Không có cơ chế “nhập đất ở vào thửa chung rồi tách ra để phân bổ đất ở” sang toàn bộ hoặc một phần đất nông nghiệp khác. Làm như vậy sẽ làm tăng diện tích đất ở mà không có quyết định cho phép chuyển mục đích và không thực hiện nghĩa vụ tài chính.
+Nếu mục tiêu là cho người nhận một thửa có đất ở, phương án đúng là: xác định phần đất ở hiện hữu của thửa 1 để tách cùng với diện tích đất trồng cây lâu năm kèm theo (nếu cần); hoặc xin chuyển mục đích phần đất trồng cây lâu năm dự kiến giao trước khi/đồng thời tách thửa. Việc tách phải đáp ứng diện tích tối thiểu đối với từng loại đất theo quyết định của UBND tỉnh nơi có đất. Điều 220 Luật Đất đai 2024
+[1]. Điều 4, Nghị quyết 254/2025/QH15
+[2]. Điều 220, Luật 31/2024/QH15</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Câu trả lời trích dẫn Điều 220 của Luật Đất đai 2024 và Điều 4 của Nghị quyết 254/2025/QH15. Tuy nhiên, không có thông tin cụ thể về nội dung của Điều 220 Luật Đất đai 2024 và Điều 4 Nghị quyết 254/2025/QH15 trong câu trả lời, do đó không thể xác định tính chính xác và hiệu lực của các điều luật này. Cần kiểm tra lại nội dung cụ thể của các điều luật để đảm bảo tính chính xác.</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="409.6" customHeight="1">
       <c r="A115" s="2" t="n">

</xml_diff>